<commit_message>
Implement student entry queue system at turnstiles
Added separate queues for each turnstile and logic to manage student placement from the queue into the grid. Updated student arrival to append to the appropriate queue and introduced a method to process and place students when possible. Also updated the simulation start hour and added comments for future improvements.

Things missing:

no refill
no interaction with some trays
</commit_message>
<xml_diff>
--- a/Modelo_RU_main/src/valores.xlsx
+++ b/Modelo_RU_main/src/valores.xlsx
@@ -17775,7 +17775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6714"/>
+  <dimension ref="A1:B7139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54394,6 +54394,3406 @@
       </c>
       <c r="B6714" t="n">
         <v>46.32881355932204</v>
+      </c>
+    </row>
+    <row r="6715">
+      <c r="A6715" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6715" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6716">
+      <c r="A6716" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6716" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6717">
+      <c r="A6717" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6717" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6718">
+      <c r="A6718" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6718" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6719">
+      <c r="A6719" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6719" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6720">
+      <c r="A6720" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6720" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6721">
+      <c r="A6721" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6721" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6722">
+      <c r="A6722" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6722" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6723">
+      <c r="A6723" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6723" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6724">
+      <c r="A6724" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6724" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6725">
+      <c r="A6725" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6725" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6726">
+      <c r="A6726" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6726" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6727">
+      <c r="A6727" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6727" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6728">
+      <c r="A6728" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6728" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6729">
+      <c r="A6729" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6729" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6730">
+      <c r="A6730" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6730" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6731">
+      <c r="A6731" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6731" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6732">
+      <c r="A6732" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6732" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6733">
+      <c r="A6733" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6733" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6734">
+      <c r="A6734" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6734" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6735">
+      <c r="A6735" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6735" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6736">
+      <c r="A6736" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6736" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6737">
+      <c r="A6737" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6737" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6738">
+      <c r="A6738" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6738" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6739">
+      <c r="A6739" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6739" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6740">
+      <c r="A6740" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6740" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6741">
+      <c r="A6741" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6741" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6742">
+      <c r="A6742" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6742" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6743">
+      <c r="A6743" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6743" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6744">
+      <c r="A6744" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6744" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6745">
+      <c r="A6745" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6745" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6746">
+      <c r="A6746" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6746" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6747">
+      <c r="A6747" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6747" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6748">
+      <c r="A6748" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6748" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6749">
+      <c r="A6749" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6749" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6750">
+      <c r="A6750" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6750" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6751">
+      <c r="A6751" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6751" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6752">
+      <c r="A6752" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6752" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6753">
+      <c r="A6753" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6753" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6754">
+      <c r="A6754" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6754" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6755">
+      <c r="A6755" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6755" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6756">
+      <c r="A6756" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6756" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6757">
+      <c r="A6757" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6757" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6758">
+      <c r="A6758" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6758" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6759">
+      <c r="A6759" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6759" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6760">
+      <c r="A6760" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6760" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6761">
+      <c r="A6761" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6761" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6762">
+      <c r="A6762" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6762" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6763">
+      <c r="A6763" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6763" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6764">
+      <c r="A6764" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6764" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6765">
+      <c r="A6765" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6765" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6766">
+      <c r="A6766" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6766" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6767">
+      <c r="A6767" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6767" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6768">
+      <c r="A6768" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6768" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6769">
+      <c r="A6769" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6769" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6770">
+      <c r="A6770" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6770" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6771">
+      <c r="A6771" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6771" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6772">
+      <c r="A6772" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6772" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6773">
+      <c r="A6773" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6773" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6774">
+      <c r="A6774" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6774" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6775">
+      <c r="A6775" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6775" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6776">
+      <c r="A6776" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6776" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6777">
+      <c r="A6777" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6777" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6778">
+      <c r="A6778" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6778" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6779">
+      <c r="A6779" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6779" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6780">
+      <c r="A6780" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6780" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6781">
+      <c r="A6781" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6781" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6782">
+      <c r="A6782" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6782" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6783">
+      <c r="A6783" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6783" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6784">
+      <c r="A6784" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6784" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6785">
+      <c r="A6785" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6785" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6786">
+      <c r="A6786" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6786" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6787">
+      <c r="A6787" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6787" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6788">
+      <c r="A6788" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6788" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6789">
+      <c r="A6789" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6789" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6790">
+      <c r="A6790" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6790" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6791">
+      <c r="A6791" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6791" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6792">
+      <c r="A6792" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6792" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6793">
+      <c r="A6793" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6793" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6794">
+      <c r="A6794" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6794" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6795">
+      <c r="A6795" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6795" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6796">
+      <c r="A6796" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6796" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6797">
+      <c r="A6797" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6797" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6798">
+      <c r="A6798" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6798" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6799">
+      <c r="A6799" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6799" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6800">
+      <c r="A6800" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6800" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6801">
+      <c r="A6801" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6801" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6802">
+      <c r="A6802" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6802" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6803">
+      <c r="A6803" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6803" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6804">
+      <c r="A6804" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6804" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6805">
+      <c r="A6805" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6805" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6806">
+      <c r="A6806" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6806" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6807">
+      <c r="A6807" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6807" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6808">
+      <c r="A6808" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6808" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6809">
+      <c r="A6809" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6809" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6810">
+      <c r="A6810" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6810" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6811">
+      <c r="A6811" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6811" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6812">
+      <c r="A6812" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6812" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6813">
+      <c r="A6813" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6813" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6814">
+      <c r="A6814" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6814" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6815">
+      <c r="A6815" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6815" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6816">
+      <c r="A6816" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6816" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6817">
+      <c r="A6817" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6817" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6818">
+      <c r="A6818" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6818" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6819">
+      <c r="A6819" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6819" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6820">
+      <c r="A6820" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6820" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6821">
+      <c r="A6821" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6821" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6822">
+      <c r="A6822" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6822" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6823">
+      <c r="A6823" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6823" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6824">
+      <c r="A6824" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6824" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6825">
+      <c r="A6825" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6825" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6826">
+      <c r="A6826" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6826" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6827">
+      <c r="A6827" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6827" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6828">
+      <c r="A6828" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6828" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6829">
+      <c r="A6829" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6829" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6830">
+      <c r="A6830" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6830" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6831">
+      <c r="A6831" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6831" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6832">
+      <c r="A6832" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6832" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6833">
+      <c r="A6833" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6833" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6834">
+      <c r="A6834" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6834" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6835">
+      <c r="A6835" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6835" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6836">
+      <c r="A6836" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6836" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6837">
+      <c r="A6837" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6837" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6838">
+      <c r="A6838" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6838" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6839">
+      <c r="A6839" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6839" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6840">
+      <c r="A6840" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6840" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6841">
+      <c r="A6841" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6841" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6842">
+      <c r="A6842" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6842" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6843">
+      <c r="A6843" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6843" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6844">
+      <c r="A6844" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6844" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6845">
+      <c r="A6845" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6845" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6846">
+      <c r="A6846" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6846" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6847">
+      <c r="A6847" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6847" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6848">
+      <c r="A6848" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6848" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6849">
+      <c r="A6849" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6849" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6850">
+      <c r="A6850" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6850" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6851">
+      <c r="A6851" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6851" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6852">
+      <c r="A6852" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6852" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6853">
+      <c r="A6853" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6853" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6854">
+      <c r="A6854" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6854" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6855">
+      <c r="A6855" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6855" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6856">
+      <c r="A6856" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6856" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6857">
+      <c r="A6857" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6857" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6858">
+      <c r="A6858" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6858" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6859">
+      <c r="A6859" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6859" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6860">
+      <c r="A6860" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6860" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6861">
+      <c r="A6861" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6861" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6862">
+      <c r="A6862" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6862" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6863">
+      <c r="A6863" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6863" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6864">
+      <c r="A6864" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6864" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6865">
+      <c r="A6865" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6865" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6866">
+      <c r="A6866" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6866" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6867">
+      <c r="A6867" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6867" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6868">
+      <c r="A6868" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6868" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6869">
+      <c r="A6869" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6869" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6870">
+      <c r="A6870" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6870" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6871">
+      <c r="A6871" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6871" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6872">
+      <c r="A6872" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6872" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6873">
+      <c r="A6873" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6873" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6874">
+      <c r="A6874" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6874" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6875">
+      <c r="A6875" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6875" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6876">
+      <c r="A6876" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6876" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6877">
+      <c r="A6877" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6877" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6878">
+      <c r="A6878" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6878" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6879">
+      <c r="A6879" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6879" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6880">
+      <c r="A6880" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6880" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6881">
+      <c r="A6881" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="B6881" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6882">
+      <c r="A6882" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6882" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6883">
+      <c r="A6883" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B6883" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6884">
+      <c r="A6884" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="B6884" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6885">
+      <c r="A6885" t="n">
+        <v>2.166666666666667</v>
+      </c>
+      <c r="B6885" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6886">
+      <c r="A6886" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6886" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6887">
+      <c r="A6887" t="n">
+        <v>3.428571428571428</v>
+      </c>
+      <c r="B6887" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6888">
+      <c r="A6888" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="B6888" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6889">
+      <c r="A6889" t="n">
+        <v>4.111111111111111</v>
+      </c>
+      <c r="B6889" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6890">
+      <c r="A6890" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6890" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6891">
+      <c r="A6891" t="n">
+        <v>4.909090909090909</v>
+      </c>
+      <c r="B6891" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6892">
+      <c r="A6892" t="n">
+        <v>4.846153846153846</v>
+      </c>
+      <c r="B6892" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6893">
+      <c r="A6893" t="n">
+        <v>5.692307692307693</v>
+      </c>
+      <c r="B6893" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6894">
+      <c r="A6894" t="n">
+        <v>6.692307692307693</v>
+      </c>
+      <c r="B6894" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6895">
+      <c r="A6895" t="n">
+        <v>6.071428571428571</v>
+      </c>
+      <c r="B6895" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6896">
+      <c r="A6896" t="n">
+        <v>6.466666666666667</v>
+      </c>
+      <c r="B6896" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6897">
+      <c r="A6897" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="B6897" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6898">
+      <c r="A6898" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="B6898" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6899">
+      <c r="A6899" t="n">
+        <v>7.833333333333333</v>
+      </c>
+      <c r="B6899" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6900">
+      <c r="A6900" t="n">
+        <v>8.666666666666666</v>
+      </c>
+      <c r="B6900" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6901">
+      <c r="A6901" t="n">
+        <v>9.058823529411764</v>
+      </c>
+      <c r="B6901" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6902">
+      <c r="A6902" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6902" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6903">
+      <c r="A6903" t="n">
+        <v>8.894736842105264</v>
+      </c>
+      <c r="B6903" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6904">
+      <c r="A6904" t="n">
+        <v>8.529411764705882</v>
+      </c>
+      <c r="B6904" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6905">
+      <c r="A6905" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6905" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6906">
+      <c r="A6906" t="n">
+        <v>8.294117647058824</v>
+      </c>
+      <c r="B6906" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6907">
+      <c r="A6907" t="n">
+        <v>8.176470588235293</v>
+      </c>
+      <c r="B6907" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6908">
+      <c r="A6908" t="n">
+        <v>8.133333333333333</v>
+      </c>
+      <c r="B6908" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6909">
+      <c r="A6909" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B6909" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6910">
+      <c r="A6910" t="n">
+        <v>7.733333333333333</v>
+      </c>
+      <c r="B6910" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6911">
+      <c r="A6911" t="n">
+        <v>8.0625</v>
+      </c>
+      <c r="B6911" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6912">
+      <c r="A6912" t="n">
+        <v>8.470588235294118</v>
+      </c>
+      <c r="B6912" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6913">
+      <c r="A6913" t="n">
+        <v>8.411764705882353</v>
+      </c>
+      <c r="B6913" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6914">
+      <c r="A6914" t="n">
+        <v>8.625</v>
+      </c>
+      <c r="B6914" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6915">
+      <c r="A6915" t="n">
+        <v>7.941176470588236</v>
+      </c>
+      <c r="B6915" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6916">
+      <c r="A6916" t="n">
+        <v>8.333333333333334</v>
+      </c>
+      <c r="B6916" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6917">
+      <c r="A6917" t="n">
+        <v>9.277777777777779</v>
+      </c>
+      <c r="B6917" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6918">
+      <c r="A6918" t="n">
+        <v>9.111111111111111</v>
+      </c>
+      <c r="B6918" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6919">
+      <c r="A6919" t="n">
+        <v>8.647058823529411</v>
+      </c>
+      <c r="B6919" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6920">
+      <c r="A6920" t="n">
+        <v>9.125</v>
+      </c>
+      <c r="B6920" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6921">
+      <c r="A6921" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="B6921" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6922">
+      <c r="A6922" t="n">
+        <v>8.625</v>
+      </c>
+      <c r="B6922" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6923">
+      <c r="A6923" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="B6923" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6924">
+      <c r="A6924" t="n">
+        <v>9</v>
+      </c>
+      <c r="B6924" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6925">
+      <c r="A6925" t="n">
+        <v>8.714285714285714</v>
+      </c>
+      <c r="B6925" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6926">
+      <c r="A6926" t="n">
+        <v>9.714285714285714</v>
+      </c>
+      <c r="B6926" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6927">
+      <c r="A6927" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6927" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6928">
+      <c r="A6928" t="n">
+        <v>10.93333333333333</v>
+      </c>
+      <c r="B6928" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6929">
+      <c r="A6929" t="n">
+        <v>11.93333333333333</v>
+      </c>
+      <c r="B6929" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6930">
+      <c r="A6930" t="n">
+        <v>10.77777777777778</v>
+      </c>
+      <c r="B6930" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6931">
+      <c r="A6931" t="n">
+        <v>11.17647058823529</v>
+      </c>
+      <c r="B6931" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6932">
+      <c r="A6932" t="n">
+        <v>10.94117647058824</v>
+      </c>
+      <c r="B6932" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6933">
+      <c r="A6933" t="n">
+        <v>11.88235294117647</v>
+      </c>
+      <c r="B6933" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6934">
+      <c r="A6934" t="n">
+        <v>12.375</v>
+      </c>
+      <c r="B6934" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6935">
+      <c r="A6935" t="n">
+        <v>10.88888888888889</v>
+      </c>
+      <c r="B6935" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6936">
+      <c r="A6936" t="n">
+        <v>11.23529411764706</v>
+      </c>
+      <c r="B6936" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6937">
+      <c r="A6937" t="n">
+        <v>12.23529411764706</v>
+      </c>
+      <c r="B6937" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6938">
+      <c r="A6938" t="n">
+        <v>12.6875</v>
+      </c>
+      <c r="B6938" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6939">
+      <c r="A6939" t="n">
+        <v>12.16666666666667</v>
+      </c>
+      <c r="B6939" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6940">
+      <c r="A6940" t="n">
+        <v>12.4375</v>
+      </c>
+      <c r="B6940" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6941">
+      <c r="A6941" t="n">
+        <v>10.70588235294118</v>
+      </c>
+      <c r="B6941" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6942">
+      <c r="A6942" t="n">
+        <v>11.58823529411765</v>
+      </c>
+      <c r="B6942" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6943">
+      <c r="A6943" t="n">
+        <v>11.88888888888889</v>
+      </c>
+      <c r="B6943" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6944">
+      <c r="A6944" t="n">
+        <v>12.83333333333333</v>
+      </c>
+      <c r="B6944" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6945">
+      <c r="A6945" t="n">
+        <v>11.94736842105263</v>
+      </c>
+      <c r="B6945" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6946">
+      <c r="A6946" t="n">
+        <v>11.89473684210526</v>
+      </c>
+      <c r="B6946" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6947">
+      <c r="A6947" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="B6947" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6948">
+      <c r="A6948" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="B6948" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6949">
+      <c r="A6949" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="B6949" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6950">
+      <c r="A6950" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="B6950" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6951">
+      <c r="A6951" t="n">
+        <v>13.52380952380952</v>
+      </c>
+      <c r="B6951" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6952">
+      <c r="A6952" t="n">
+        <v>13.21739130434783</v>
+      </c>
+      <c r="B6952" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6953">
+      <c r="A6953" t="n">
+        <v>14.1304347826087</v>
+      </c>
+      <c r="B6953" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6954">
+      <c r="A6954" t="n">
+        <v>14.34782608695652</v>
+      </c>
+      <c r="B6954" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6955">
+      <c r="A6955" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="B6955" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6956">
+      <c r="A6956" t="n">
+        <v>14.42307692307692</v>
+      </c>
+      <c r="B6956" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6957">
+      <c r="A6957" t="n">
+        <v>15.04</v>
+      </c>
+      <c r="B6957" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6958">
+      <c r="A6958" t="n">
+        <v>14.07692307692308</v>
+      </c>
+      <c r="B6958" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6959">
+      <c r="A6959" t="n">
+        <v>14.44444444444444</v>
+      </c>
+      <c r="B6959" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6960">
+      <c r="A6960" t="n">
+        <v>15.40740740740741</v>
+      </c>
+      <c r="B6960" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6961">
+      <c r="A6961" t="n">
+        <v>16.40740740740741</v>
+      </c>
+      <c r="B6961" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6962">
+      <c r="A6962" t="n">
+        <v>15.66666666666667</v>
+      </c>
+      <c r="B6962" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6963">
+      <c r="A6963" t="n">
+        <v>16.56666666666667</v>
+      </c>
+      <c r="B6963" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6964">
+      <c r="A6964" t="n">
+        <v>17</v>
+      </c>
+      <c r="B6964" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6965">
+      <c r="A6965" t="n">
+        <v>17.48387096774194</v>
+      </c>
+      <c r="B6965" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6966">
+      <c r="A6966" t="n">
+        <v>17.875</v>
+      </c>
+      <c r="B6966" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6967">
+      <c r="A6967" t="n">
+        <v>18.27272727272727</v>
+      </c>
+      <c r="B6967" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6968">
+      <c r="A6968" t="n">
+        <v>18.14285714285714</v>
+      </c>
+      <c r="B6968" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6969">
+      <c r="A6969" t="n">
+        <v>19.08571428571429</v>
+      </c>
+      <c r="B6969" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6970">
+      <c r="A6970" t="n">
+        <v>20.08571428571429</v>
+      </c>
+      <c r="B6970" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6971">
+      <c r="A6971" t="n">
+        <v>19.94594594594595</v>
+      </c>
+      <c r="B6971" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6972">
+      <c r="A6972" t="n">
+        <v>20.37837837837838</v>
+      </c>
+      <c r="B6972" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6973">
+      <c r="A6973" t="n">
+        <v>21.36111111111111</v>
+      </c>
+      <c r="B6973" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6974">
+      <c r="A6974" t="n">
+        <v>21.18421052631579</v>
+      </c>
+      <c r="B6974" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6975">
+      <c r="A6975" t="n">
+        <v>21.56410256410257</v>
+      </c>
+      <c r="B6975" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6976">
+      <c r="A6976" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="B6976" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6977">
+      <c r="A6977" t="n">
+        <v>21.56756756756757</v>
+      </c>
+      <c r="B6977" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6978">
+      <c r="A6978" t="n">
+        <v>21.47222222222222</v>
+      </c>
+      <c r="B6978" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6979">
+      <c r="A6979" t="n">
+        <v>21.83783783783784</v>
+      </c>
+      <c r="B6979" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6980">
+      <c r="A6980" t="n">
+        <v>22.81081081081081</v>
+      </c>
+      <c r="B6980" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6981">
+      <c r="A6981" t="n">
+        <v>23.81081081081081</v>
+      </c>
+      <c r="B6981" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6982">
+      <c r="A6982" t="n">
+        <v>24.81081081081081</v>
+      </c>
+      <c r="B6982" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6983">
+      <c r="A6983" t="n">
+        <v>25.32432432432432</v>
+      </c>
+      <c r="B6983" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6984">
+      <c r="A6984" t="n">
+        <v>25.60526315789474</v>
+      </c>
+      <c r="B6984" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6985">
+      <c r="A6985" t="n">
+        <v>26.57894736842105</v>
+      </c>
+      <c r="B6985" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6986">
+      <c r="A6986" t="n">
+        <v>27.57894736842105</v>
+      </c>
+      <c r="B6986" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6987">
+      <c r="A6987" t="n">
+        <v>27.84615384615385</v>
+      </c>
+      <c r="B6987" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6988">
+      <c r="A6988" t="n">
+        <v>28.82051282051282</v>
+      </c>
+      <c r="B6988" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6989">
+      <c r="A6989" t="n">
+        <v>29.075</v>
+      </c>
+      <c r="B6989" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6990">
+      <c r="A6990" t="n">
+        <v>29.31707317073171</v>
+      </c>
+      <c r="B6990" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6991">
+      <c r="A6991" t="n">
+        <v>30.29268292682927</v>
+      </c>
+      <c r="B6991" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6992">
+      <c r="A6992" t="n">
+        <v>30.95</v>
+      </c>
+      <c r="B6992" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6993">
+      <c r="A6993" t="n">
+        <v>31.95</v>
+      </c>
+      <c r="B6993" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6994">
+      <c r="A6994" t="n">
+        <v>32.14634146341464</v>
+      </c>
+      <c r="B6994" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6995">
+      <c r="A6995" t="n">
+        <v>33.1219512195122</v>
+      </c>
+      <c r="B6995" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6996">
+      <c r="A6996" t="n">
+        <v>33.30952380952381</v>
+      </c>
+      <c r="B6996" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6997">
+      <c r="A6997" t="n">
+        <v>33.48837209302326</v>
+      </c>
+      <c r="B6997" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6998">
+      <c r="A6998" t="n">
+        <v>33.69047619047619</v>
+      </c>
+      <c r="B6998" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6999">
+      <c r="A6999" t="n">
+        <v>34.69047619047619</v>
+      </c>
+      <c r="B6999" t="n">
+        <v>0.1978021978021978</v>
+      </c>
+    </row>
+    <row r="7000">
+      <c r="A7000" t="n">
+        <v>34.86046511627907</v>
+      </c>
+      <c r="B7000" t="n">
+        <v>0.391304347826087</v>
+      </c>
+    </row>
+    <row r="7001">
+      <c r="A7001" t="n">
+        <v>35.83720930232558</v>
+      </c>
+      <c r="B7001" t="n">
+        <v>0.391304347826087</v>
+      </c>
+    </row>
+    <row r="7002">
+      <c r="A7002" t="n">
+        <v>36.41860465116279</v>
+      </c>
+      <c r="B7002" t="n">
+        <v>0.3870967741935484</v>
+      </c>
+    </row>
+    <row r="7003">
+      <c r="A7003" t="n">
+        <v>36.54545454545455</v>
+      </c>
+      <c r="B7003" t="n">
+        <v>0.574468085106383</v>
+      </c>
+    </row>
+    <row r="7004">
+      <c r="A7004" t="n">
+        <v>37.52272727272727</v>
+      </c>
+      <c r="B7004" t="n">
+        <v>0.574468085106383</v>
+      </c>
+    </row>
+    <row r="7005">
+      <c r="A7005" t="n">
+        <v>38.52272727272727</v>
+      </c>
+      <c r="B7005" t="n">
+        <v>0.574468085106383</v>
+      </c>
+    </row>
+    <row r="7006">
+      <c r="A7006" t="n">
+        <v>38.64444444444445</v>
+      </c>
+      <c r="B7006" t="n">
+        <v>0.5684210526315789</v>
+      </c>
+    </row>
+    <row r="7007">
+      <c r="A7007" t="n">
+        <v>39.62222222222222</v>
+      </c>
+      <c r="B7007" t="n">
+        <v>0.5684210526315789</v>
+      </c>
+    </row>
+    <row r="7008">
+      <c r="A7008" t="n">
+        <v>40.62222222222222</v>
+      </c>
+      <c r="B7008" t="n">
+        <v>0.5684210526315789</v>
+      </c>
+    </row>
+    <row r="7009">
+      <c r="A7009" t="n">
+        <v>40.71739130434783</v>
+      </c>
+      <c r="B7009" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+    </row>
+    <row r="7010">
+      <c r="A7010" t="n">
+        <v>41.69565217391305</v>
+      </c>
+      <c r="B7010" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+    </row>
+    <row r="7011">
+      <c r="A7011" t="n">
+        <v>42.69565217391305</v>
+      </c>
+      <c r="B7011" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+    </row>
+    <row r="7012">
+      <c r="A7012" t="n">
+        <v>42.76595744680851</v>
+      </c>
+      <c r="B7012" t="n">
+        <v>0.7628865979381443</v>
+      </c>
+    </row>
+    <row r="7013">
+      <c r="A7013" t="n">
+        <v>42.24444444444445</v>
+      </c>
+      <c r="B7013" t="n">
+        <v>0.9690721649484536</v>
+      </c>
+    </row>
+    <row r="7014">
+      <c r="A7014" t="n">
+        <v>42.54545454545455</v>
+      </c>
+      <c r="B7014" t="n">
+        <v>0.9690721649484536</v>
+      </c>
+    </row>
+    <row r="7015">
+      <c r="A7015" t="n">
+        <v>43.54545454545455</v>
+      </c>
+      <c r="B7015" t="n">
+        <v>0.9690721649484536</v>
+      </c>
+    </row>
+    <row r="7016">
+      <c r="A7016" t="n">
+        <v>41.77777777777778</v>
+      </c>
+      <c r="B7016" t="n">
+        <v>1.171717171717172</v>
+      </c>
+    </row>
+    <row r="7017">
+      <c r="A7017" t="n">
+        <v>42.73333333333333</v>
+      </c>
+      <c r="B7017" t="n">
+        <v>1.171717171717172</v>
+      </c>
+    </row>
+    <row r="7018">
+      <c r="A7018" t="n">
+        <v>43.73333333333333</v>
+      </c>
+      <c r="B7018" t="n">
+        <v>1.171717171717172</v>
+      </c>
+    </row>
+    <row r="7019">
+      <c r="A7019" t="n">
+        <v>43.76086956521739</v>
+      </c>
+      <c r="B7019" t="n">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="7020">
+      <c r="A7020" t="n">
+        <v>44.73913043478261</v>
+      </c>
+      <c r="B7020" t="n">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="7021">
+      <c r="A7021" t="n">
+        <v>45.25</v>
+      </c>
+      <c r="B7021" t="n">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="7022">
+      <c r="A7022" t="n">
+        <v>44.23913043478261</v>
+      </c>
+      <c r="B7022" t="n">
+        <v>1.450980392156863</v>
+      </c>
+    </row>
+    <row r="7023">
+      <c r="A7023" t="n">
+        <v>45.19565217391305</v>
+      </c>
+      <c r="B7023" t="n">
+        <v>1.450980392156863</v>
+      </c>
+    </row>
+    <row r="7024">
+      <c r="A7024" t="n">
+        <v>46.19565217391305</v>
+      </c>
+      <c r="B7024" t="n">
+        <v>1.450980392156863</v>
+      </c>
+    </row>
+    <row r="7025">
+      <c r="A7025" t="n">
+        <v>47.19565217391305</v>
+      </c>
+      <c r="B7025" t="n">
+        <v>1.450980392156863</v>
+      </c>
+    </row>
+    <row r="7026">
+      <c r="A7026" t="n">
+        <v>47.17021276595744</v>
+      </c>
+      <c r="B7026" t="n">
+        <v>1.58252427184466</v>
+      </c>
+    </row>
+    <row r="7027">
+      <c r="A7027" t="n">
+        <v>48.14893617021276</v>
+      </c>
+      <c r="B7027" t="n">
+        <v>1.766990291262136</v>
+      </c>
+    </row>
+    <row r="7028">
+      <c r="A7028" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="B7028" t="n">
+        <v>1.766990291262136</v>
+      </c>
+    </row>
+    <row r="7029">
+      <c r="A7029" t="n">
+        <v>48.32608695652174</v>
+      </c>
+      <c r="B7029" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="7030">
+      <c r="A7030" t="n">
+        <v>48.25531914893617</v>
+      </c>
+      <c r="B7030" t="n">
+        <v>1.733333333333333</v>
+      </c>
+    </row>
+    <row r="7031">
+      <c r="A7031" t="n">
+        <v>48.60869565217391</v>
+      </c>
+      <c r="B7031" t="n">
+        <v>1.733333333333333</v>
+      </c>
+    </row>
+    <row r="7032">
+      <c r="A7032" t="n">
+        <v>49.02222222222223</v>
+      </c>
+      <c r="B7032" t="n">
+        <v>1.733333333333333</v>
+      </c>
+    </row>
+    <row r="7033">
+      <c r="A7033" t="n">
+        <v>48.93478260869565</v>
+      </c>
+      <c r="B7033" t="n">
+        <v>1.716981132075472</v>
+      </c>
+    </row>
+    <row r="7034">
+      <c r="A7034" t="n">
+        <v>49.91304347826087</v>
+      </c>
+      <c r="B7034" t="n">
+        <v>1.915094339622641</v>
+      </c>
+    </row>
+    <row r="7035">
+      <c r="A7035" t="n">
+        <v>50.91304347826087</v>
+      </c>
+      <c r="B7035" t="n">
+        <v>1.915094339622641</v>
+      </c>
+    </row>
+    <row r="7036">
+      <c r="A7036" t="n">
+        <v>50.80851063829788</v>
+      </c>
+      <c r="B7036" t="n">
+        <v>2.065420560747663</v>
+      </c>
+    </row>
+    <row r="7037">
+      <c r="A7037" t="n">
+        <v>50.70833333333334</v>
+      </c>
+      <c r="B7037" t="n">
+        <v>2.222222222222222</v>
+      </c>
+    </row>
+    <row r="7038">
+      <c r="A7038" t="n">
+        <v>51.6875</v>
+      </c>
+      <c r="B7038" t="n">
+        <v>2.222222222222222</v>
+      </c>
+    </row>
+    <row r="7039">
+      <c r="A7039" t="n">
+        <v>52.6875</v>
+      </c>
+      <c r="B7039" t="n">
+        <v>2.222222222222222</v>
+      </c>
+    </row>
+    <row r="7040">
+      <c r="A7040" t="n">
+        <v>53.6875</v>
+      </c>
+      <c r="B7040" t="n">
+        <v>2.222222222222222</v>
+      </c>
+    </row>
+    <row r="7041">
+      <c r="A7041" t="n">
+        <v>53.57142857142857</v>
+      </c>
+      <c r="B7041" t="n">
+        <v>2.201834862385321</v>
+      </c>
+    </row>
+    <row r="7042">
+      <c r="A7042" t="n">
+        <v>54.55102040816327</v>
+      </c>
+      <c r="B7042" t="n">
+        <v>2.201834862385321</v>
+      </c>
+    </row>
+    <row r="7043">
+      <c r="A7043" t="n">
+        <v>54.44</v>
+      </c>
+      <c r="B7043" t="n">
+        <v>2.181818181818182</v>
+      </c>
+    </row>
+    <row r="7044">
+      <c r="A7044" t="n">
+        <v>55.42</v>
+      </c>
+      <c r="B7044" t="n">
+        <v>2.181818181818182</v>
+      </c>
+    </row>
+    <row r="7045">
+      <c r="A7045" t="n">
+        <v>55.31372549019608</v>
+      </c>
+      <c r="B7045" t="n">
+        <v>2.162162162162162</v>
+      </c>
+    </row>
+    <row r="7046">
+      <c r="A7046" t="n">
+        <v>55.86</v>
+      </c>
+      <c r="B7046" t="n">
+        <v>2.162162162162162</v>
+      </c>
+    </row>
+    <row r="7047">
+      <c r="A7047" t="n">
+        <v>56.86</v>
+      </c>
+      <c r="B7047" t="n">
+        <v>2.162162162162162</v>
+      </c>
+    </row>
+    <row r="7048">
+      <c r="A7048" t="n">
+        <v>56.72549019607843</v>
+      </c>
+      <c r="B7048" t="n">
+        <v>2.142857142857143</v>
+      </c>
+    </row>
+    <row r="7049">
+      <c r="A7049" t="n">
+        <v>56.59615384615385</v>
+      </c>
+      <c r="B7049" t="n">
+        <v>2.123893805309735</v>
+      </c>
+    </row>
+    <row r="7050">
+      <c r="A7050" t="n">
+        <v>56.49056603773585</v>
+      </c>
+      <c r="B7050" t="n">
+        <v>2.105263157894737</v>
+      </c>
+    </row>
+    <row r="7051">
+      <c r="A7051" t="n">
+        <v>57.47169811320754</v>
+      </c>
+      <c r="B7051" t="n">
+        <v>2.105263157894737</v>
+      </c>
+    </row>
+    <row r="7052">
+      <c r="A7052" t="n">
+        <v>57.36538461538461</v>
+      </c>
+      <c r="B7052" t="n">
+        <v>2.105263157894737</v>
+      </c>
+    </row>
+    <row r="7053">
+      <c r="A7053" t="n">
+        <v>56.2037037037037</v>
+      </c>
+      <c r="B7053" t="n">
+        <v>2.068965517241379</v>
+      </c>
+    </row>
+    <row r="7054">
+      <c r="A7054" t="n">
+        <v>55.40384615384615</v>
+      </c>
+      <c r="B7054" t="n">
+        <v>2.068965517241379</v>
+      </c>
+    </row>
+    <row r="7055">
+      <c r="A7055" t="n">
+        <v>55.33962264150944</v>
+      </c>
+      <c r="B7055" t="n">
+        <v>2.051282051282051</v>
+      </c>
+    </row>
+    <row r="7056">
+      <c r="A7056" t="n">
+        <v>54.3921568627451</v>
+      </c>
+      <c r="B7056" t="n">
+        <v>2.051282051282051</v>
+      </c>
+    </row>
+    <row r="7057">
+      <c r="A7057" t="n">
+        <v>53.30188679245283</v>
+      </c>
+      <c r="B7057" t="n">
+        <v>2.168067226890756</v>
+      </c>
+    </row>
+    <row r="7058">
+      <c r="A7058" t="n">
+        <v>54.26415094339622</v>
+      </c>
+      <c r="B7058" t="n">
+        <v>2.344537815126051</v>
+      </c>
+    </row>
+    <row r="7059">
+      <c r="A7059" t="n">
+        <v>54.07692307692308</v>
+      </c>
+      <c r="B7059" t="n">
+        <v>2.344537815126051</v>
+      </c>
+    </row>
+    <row r="7060">
+      <c r="A7060" t="n">
+        <v>53.05769230769231</v>
+      </c>
+      <c r="B7060" t="n">
+        <v>2.325</v>
+      </c>
+    </row>
+    <row r="7061">
+      <c r="A7061" t="n">
+        <v>54.03846153846154</v>
+      </c>
+      <c r="B7061" t="n">
+        <v>2.325</v>
+      </c>
+    </row>
+    <row r="7062">
+      <c r="A7062" t="n">
+        <v>55.03846153846154</v>
+      </c>
+      <c r="B7062" t="n">
+        <v>2.325</v>
+      </c>
+    </row>
+    <row r="7063">
+      <c r="A7063" t="n">
+        <v>56.03846153846154</v>
+      </c>
+      <c r="B7063" t="n">
+        <v>2.325</v>
+      </c>
+    </row>
+    <row r="7064">
+      <c r="A7064" t="n">
+        <v>54.92592592592592</v>
+      </c>
+      <c r="B7064" t="n">
+        <v>2.459016393442623</v>
+      </c>
+    </row>
+    <row r="7065">
+      <c r="A7065" t="n">
+        <v>55.88888888888889</v>
+      </c>
+      <c r="B7065" t="n">
+        <v>2.639344262295082</v>
+      </c>
+    </row>
+    <row r="7066">
+      <c r="A7066" t="n">
+        <v>56.88888888888889</v>
+      </c>
+      <c r="B7066" t="n">
+        <v>2.639344262295082</v>
+      </c>
+    </row>
+    <row r="7067">
+      <c r="A7067" t="n">
+        <v>54.87272727272727</v>
+      </c>
+      <c r="B7067" t="n">
+        <v>2.596774193548387</v>
+      </c>
+    </row>
+    <row r="7068">
+      <c r="A7068" t="n">
+        <v>55.83636363636364</v>
+      </c>
+      <c r="B7068" t="n">
+        <v>2.596774193548387</v>
+      </c>
+    </row>
+    <row r="7069">
+      <c r="A7069" t="n">
+        <v>56.83636363636364</v>
+      </c>
+      <c r="B7069" t="n">
+        <v>2.596774193548387</v>
+      </c>
+    </row>
+    <row r="7070">
+      <c r="A7070" t="n">
+        <v>57.83636363636364</v>
+      </c>
+      <c r="B7070" t="n">
+        <v>2.741935483870968</v>
+      </c>
+    </row>
+    <row r="7071">
+      <c r="A7071" t="n">
+        <v>58.83636363636364</v>
+      </c>
+      <c r="B7071" t="n">
+        <v>2.741935483870968</v>
+      </c>
+    </row>
+    <row r="7072">
+      <c r="A7072" t="n">
+        <v>58.76785714285715</v>
+      </c>
+      <c r="B7072" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="7073">
+      <c r="A7073" t="n">
+        <v>59.41818181818182</v>
+      </c>
+      <c r="B7073" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="7074">
+      <c r="A7074" t="n">
+        <v>60.41818181818182</v>
+      </c>
+      <c r="B7074" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="7075">
+      <c r="A7075" t="n">
+        <v>60.32142857142857</v>
+      </c>
+      <c r="B7075" t="n">
+        <v>2.96031746031746</v>
+      </c>
+    </row>
+    <row r="7076">
+      <c r="A7076" t="n">
+        <v>59.73214285714285</v>
+      </c>
+      <c r="B7076" t="n">
+        <v>3.086614173228346</v>
+      </c>
+    </row>
+    <row r="7077">
+      <c r="A7077" t="n">
+        <v>60.71428571428572</v>
+      </c>
+      <c r="B7077" t="n">
+        <v>3.086614173228346</v>
+      </c>
+    </row>
+    <row r="7078">
+      <c r="A7078" t="n">
+        <v>61.71428571428572</v>
+      </c>
+      <c r="B7078" t="n">
+        <v>3.275590551181102</v>
+      </c>
+    </row>
+    <row r="7079">
+      <c r="A7079" t="n">
+        <v>62.36363636363637</v>
+      </c>
+      <c r="B7079" t="n">
+        <v>3.275590551181102</v>
+      </c>
+    </row>
+    <row r="7080">
+      <c r="A7080" t="n">
+        <v>63.36363636363637</v>
+      </c>
+      <c r="B7080" t="n">
+        <v>3.275590551181102</v>
+      </c>
+    </row>
+    <row r="7081">
+      <c r="A7081" t="n">
+        <v>63.21428571428572</v>
+      </c>
+      <c r="B7081" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="7082">
+      <c r="A7082" t="n">
+        <v>64.19642857142857</v>
+      </c>
+      <c r="B7082" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="7083">
+      <c r="A7083" t="n">
+        <v>65.19642857142857</v>
+      </c>
+      <c r="B7083" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="7084">
+      <c r="A7084" t="n">
+        <v>65.03508771929825</v>
+      </c>
+      <c r="B7084" t="n">
+        <v>3.224806201550388</v>
+      </c>
+    </row>
+    <row r="7085">
+      <c r="A7085" t="n">
+        <v>64.87931034482759</v>
+      </c>
+      <c r="B7085" t="n">
+        <v>3.346153846153846</v>
+      </c>
+    </row>
+    <row r="7086">
+      <c r="A7086" t="n">
+        <v>64.59649122807018</v>
+      </c>
+      <c r="B7086" t="n">
+        <v>3.346153846153846</v>
+      </c>
+    </row>
+    <row r="7087">
+      <c r="A7087" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="B7087" t="n">
+        <v>3.476923076923077</v>
+      </c>
+    </row>
+    <row r="7088">
+      <c r="A7088" t="n">
+        <v>64.16363636363636</v>
+      </c>
+      <c r="B7088" t="n">
+        <v>3.476923076923077</v>
+      </c>
+    </row>
+    <row r="7089">
+      <c r="A7089" t="n">
+        <v>64.44444444444444</v>
+      </c>
+      <c r="B7089" t="n">
+        <v>3.607692307692308</v>
+      </c>
+    </row>
+    <row r="7090">
+      <c r="A7090" t="n">
+        <v>65.44444444444444</v>
+      </c>
+      <c r="B7090" t="n">
+        <v>3.607692307692308</v>
+      </c>
+    </row>
+    <row r="7091">
+      <c r="A7091" t="n">
+        <v>66.44444444444444</v>
+      </c>
+      <c r="B7091" t="n">
+        <v>3.607692307692308</v>
+      </c>
+    </row>
+    <row r="7092">
+      <c r="A7092" t="n">
+        <v>67.44444444444444</v>
+      </c>
+      <c r="B7092" t="n">
+        <v>3.607692307692308</v>
+      </c>
+    </row>
+    <row r="7093">
+      <c r="A7093" t="n">
+        <v>68.44444444444444</v>
+      </c>
+      <c r="B7093" t="n">
+        <v>3.607692307692308</v>
+      </c>
+    </row>
+    <row r="7094">
+      <c r="A7094" t="n">
+        <v>68.18181818181819</v>
+      </c>
+      <c r="B7094" t="n">
+        <v>3.725190839694656</v>
+      </c>
+    </row>
+    <row r="7095">
+      <c r="A7095" t="n">
+        <v>69.16363636363636</v>
+      </c>
+      <c r="B7095" t="n">
+        <v>3.725190839694656</v>
+      </c>
+    </row>
+    <row r="7096">
+      <c r="A7096" t="n">
+        <v>70.16363636363636</v>
+      </c>
+      <c r="B7096" t="n">
+        <v>3.885496183206107</v>
+      </c>
+    </row>
+    <row r="7097">
+      <c r="A7097" t="n">
+        <v>70.07407407407408</v>
+      </c>
+      <c r="B7097" t="n">
+        <v>3.885496183206107</v>
+      </c>
+    </row>
+    <row r="7098">
+      <c r="A7098" t="n">
+        <v>71.07407407407408</v>
+      </c>
+      <c r="B7098" t="n">
+        <v>3.885496183206107</v>
+      </c>
+    </row>
+    <row r="7099">
+      <c r="A7099" t="n">
+        <v>72.07407407407408</v>
+      </c>
+      <c r="B7099" t="n">
+        <v>3.885496183206107</v>
+      </c>
+    </row>
+    <row r="7100">
+      <c r="A7100" t="n">
+        <v>73.07407407407408</v>
+      </c>
+      <c r="B7100" t="n">
+        <v>4.137404580152672</v>
+      </c>
+    </row>
+    <row r="7101">
+      <c r="A7101" t="n">
+        <v>74.07407407407408</v>
+      </c>
+      <c r="B7101" t="n">
+        <v>4.137404580152672</v>
+      </c>
+    </row>
+    <row r="7102">
+      <c r="A7102" t="n">
+        <v>75.07407407407408</v>
+      </c>
+      <c r="B7102" t="n">
+        <v>4.137404580152672</v>
+      </c>
+    </row>
+    <row r="7103">
+      <c r="A7103" t="n">
+        <v>73.42592592592592</v>
+      </c>
+      <c r="B7103" t="n">
+        <v>4.106060606060606</v>
+      </c>
+    </row>
+    <row r="7104">
+      <c r="A7104" t="n">
+        <v>74.4074074074074</v>
+      </c>
+      <c r="B7104" t="n">
+        <v>4.106060606060606</v>
+      </c>
+    </row>
+    <row r="7105">
+      <c r="A7105" t="n">
+        <v>74.03636363636363</v>
+      </c>
+      <c r="B7105" t="n">
+        <v>4.075187969924812</v>
+      </c>
+    </row>
+    <row r="7106">
+      <c r="A7106" t="n">
+        <v>73.98148148148148</v>
+      </c>
+      <c r="B7106" t="n">
+        <v>4.360902255639098</v>
+      </c>
+    </row>
+    <row r="7107">
+      <c r="A7107" t="n">
+        <v>74.98148148148148</v>
+      </c>
+      <c r="B7107" t="n">
+        <v>4.360902255639098</v>
+      </c>
+    </row>
+    <row r="7108">
+      <c r="A7108" t="n">
+        <v>75.62264150943396</v>
+      </c>
+      <c r="B7108" t="n">
+        <v>4.541353383458647</v>
+      </c>
+    </row>
+    <row r="7109">
+      <c r="A7109" t="n">
+        <v>74.52830188679245</v>
+      </c>
+      <c r="B7109" t="n">
+        <v>4.507462686567164</v>
+      </c>
+    </row>
+    <row r="7110">
+      <c r="A7110" t="n">
+        <v>74.11111111111111</v>
+      </c>
+      <c r="B7110" t="n">
+        <v>4.474074074074074</v>
+      </c>
+    </row>
+    <row r="7111">
+      <c r="A7111" t="n">
+        <v>75.0925925925926</v>
+      </c>
+      <c r="B7111" t="n">
+        <v>4.474074074074074</v>
+      </c>
+    </row>
+    <row r="7112">
+      <c r="A7112" t="n">
+        <v>76.0925925925926</v>
+      </c>
+      <c r="B7112" t="n">
+        <v>4.474074074074074</v>
+      </c>
+    </row>
+    <row r="7113">
+      <c r="A7113" t="n">
+        <v>74.53703703703704</v>
+      </c>
+      <c r="B7113" t="n">
+        <v>4.573529411764706</v>
+      </c>
+    </row>
+    <row r="7114">
+      <c r="A7114" t="n">
+        <v>75.51851851851852</v>
+      </c>
+      <c r="B7114" t="n">
+        <v>4.573529411764706</v>
+      </c>
+    </row>
+    <row r="7115">
+      <c r="A7115" t="n">
+        <v>76.51851851851852</v>
+      </c>
+      <c r="B7115" t="n">
+        <v>4.573529411764706</v>
+      </c>
+    </row>
+    <row r="7116">
+      <c r="A7116" t="n">
+        <v>76.60377358490567</v>
+      </c>
+      <c r="B7116" t="n">
+        <v>4.573529411764706</v>
+      </c>
+    </row>
+    <row r="7117">
+      <c r="A7117" t="n">
+        <v>76.16666666666667</v>
+      </c>
+      <c r="B7117" t="n">
+        <v>4.54014598540146</v>
+      </c>
+    </row>
+    <row r="7118">
+      <c r="A7118" t="n">
+        <v>76.20754716981132</v>
+      </c>
+      <c r="B7118" t="n">
+        <v>4.700729927007299</v>
+      </c>
+    </row>
+    <row r="7119">
+      <c r="A7119" t="n">
+        <v>74.23529411764706</v>
+      </c>
+      <c r="B7119" t="n">
+        <v>4.700729927007299</v>
+      </c>
+    </row>
+    <row r="7120">
+      <c r="A7120" t="n">
+        <v>75.23529411764706</v>
+      </c>
+      <c r="B7120" t="n">
+        <v>5.116788321167883</v>
+      </c>
+    </row>
+    <row r="7121">
+      <c r="A7121" t="n">
+        <v>74</v>
+      </c>
+      <c r="B7121" t="n">
+        <v>5.079710144927536</v>
+      </c>
+    </row>
+    <row r="7122">
+      <c r="A7122" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="B7122" t="n">
+        <v>5.079710144927536</v>
+      </c>
+    </row>
+    <row r="7123">
+      <c r="A7123" t="n">
+        <v>75.38</v>
+      </c>
+      <c r="B7123" t="n">
+        <v>5.079710144927536</v>
+      </c>
+    </row>
+    <row r="7124">
+      <c r="A7124" t="n">
+        <v>74.88235294117646</v>
+      </c>
+      <c r="B7124" t="n">
+        <v>5.043165467625899</v>
+      </c>
+    </row>
+    <row r="7125">
+      <c r="A7125" t="n">
+        <v>75.86274509803921</v>
+      </c>
+      <c r="B7125" t="n">
+        <v>5.043165467625899</v>
+      </c>
+    </row>
+    <row r="7126">
+      <c r="A7126" t="n">
+        <v>76.86274509803921</v>
+      </c>
+      <c r="B7126" t="n">
+        <v>5.043165467625899</v>
+      </c>
+    </row>
+    <row r="7127">
+      <c r="A7127" t="n">
+        <v>77.86274509803921</v>
+      </c>
+      <c r="B7127" t="n">
+        <v>5.302158273381295</v>
+      </c>
+    </row>
+    <row r="7128">
+      <c r="A7128" t="n">
+        <v>78.86274509803921</v>
+      </c>
+      <c r="B7128" t="n">
+        <v>5.302158273381295</v>
+      </c>
+    </row>
+    <row r="7129">
+      <c r="A7129" t="n">
+        <v>79.86274509803921</v>
+      </c>
+      <c r="B7129" t="n">
+        <v>5.431654676258993</v>
+      </c>
+    </row>
+    <row r="7130">
+      <c r="A7130" t="n">
+        <v>79.30769230769231</v>
+      </c>
+      <c r="B7130" t="n">
+        <v>5.392857142857143</v>
+      </c>
+    </row>
+    <row r="7131">
+      <c r="A7131" t="n">
+        <v>80.28846153846153</v>
+      </c>
+      <c r="B7131" t="n">
+        <v>5.714285714285714</v>
+      </c>
+    </row>
+    <row r="7132">
+      <c r="A7132" t="n">
+        <v>81.28846153846153</v>
+      </c>
+      <c r="B7132" t="n">
+        <v>5.964285714285714</v>
+      </c>
+    </row>
+    <row r="7133">
+      <c r="A7133" t="n">
+        <v>82.28846153846153</v>
+      </c>
+      <c r="B7133" t="n">
+        <v>5.964285714285714</v>
+      </c>
+    </row>
+    <row r="7134">
+      <c r="A7134" t="n">
+        <v>83.28846153846153</v>
+      </c>
+      <c r="B7134" t="n">
+        <v>5.964285714285714</v>
+      </c>
+    </row>
+    <row r="7135">
+      <c r="A7135" t="n">
+        <v>84.28846153846153</v>
+      </c>
+      <c r="B7135" t="n">
+        <v>5.964285714285714</v>
+      </c>
+    </row>
+    <row r="7136">
+      <c r="A7136" t="n">
+        <v>83.67924528301887</v>
+      </c>
+      <c r="B7136" t="n">
+        <v>6.049645390070922</v>
+      </c>
+    </row>
+    <row r="7137">
+      <c r="A7137" t="n">
+        <v>83</v>
+      </c>
+      <c r="B7137" t="n">
+        <v>6.049645390070922</v>
+      </c>
+    </row>
+    <row r="7138">
+      <c r="A7138" t="n">
+        <v>84</v>
+      </c>
+      <c r="B7138" t="n">
+        <v>6.382978723404255</v>
+      </c>
+    </row>
+    <row r="7139">
+      <c r="A7139" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7139" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Colocadas as interações com sobremesa e condimentos
</commit_message>
<xml_diff>
--- a/Modelo_RU_main/src/valores.xlsx
+++ b/Modelo_RU_main/src/valores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7780"/>
+  <dimension ref="A1:B7783"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62656,6 +62656,30 @@
         <v>26.12738853503185</v>
       </c>
     </row>
+    <row r="7781">
+      <c r="A7781" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7781" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7782">
+      <c r="A7782" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7782" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7783">
+      <c r="A7783" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7783" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Modelo rodando sem visualização. Para reverter, descomente em main.py
</commit_message>
<xml_diff>
--- a/Modelo_RU_main/src/valores.xlsx
+++ b/Modelo_RU_main/src/valores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7783"/>
+  <dimension ref="A1:B8327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62680,6 +62680,4358 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7784">
+      <c r="A7784" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7784" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7785">
+      <c r="A7785" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7785" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7786">
+      <c r="A7786" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7786" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7787">
+      <c r="A7787" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7787" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7788">
+      <c r="A7788" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7788" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7789">
+      <c r="A7789" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7789" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7790">
+      <c r="A7790" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7790" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7791">
+      <c r="A7791" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7791" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7792">
+      <c r="A7792" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7792" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7793">
+      <c r="A7793" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7793" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7794">
+      <c r="A7794" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7794" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7795">
+      <c r="A7795" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7795" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7796">
+      <c r="A7796" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7796" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7797">
+      <c r="A7797" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7797" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7798">
+      <c r="A7798" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7798" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7799">
+      <c r="A7799" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7799" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7800">
+      <c r="A7800" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7800" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7801">
+      <c r="A7801" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7801" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7802">
+      <c r="A7802" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7802" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7803">
+      <c r="A7803" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7803" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7804">
+      <c r="A7804" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7804" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7805">
+      <c r="A7805" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7805" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7806">
+      <c r="A7806" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7806" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7807">
+      <c r="A7807" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7807" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7808">
+      <c r="A7808" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7808" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7809">
+      <c r="A7809" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7809" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7810">
+      <c r="A7810" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7810" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7811">
+      <c r="A7811" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7811" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7812">
+      <c r="A7812" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7812" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7813">
+      <c r="A7813" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7813" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7814">
+      <c r="A7814" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7814" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7815">
+      <c r="A7815" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7815" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7816">
+      <c r="A7816" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7816" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7817">
+      <c r="A7817" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7817" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7818">
+      <c r="A7818" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7818" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7819">
+      <c r="A7819" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7819" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7820">
+      <c r="A7820" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7820" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7821">
+      <c r="A7821" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7821" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7822">
+      <c r="A7822" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7822" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7823">
+      <c r="A7823" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7823" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7824">
+      <c r="A7824" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7824" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7825">
+      <c r="A7825" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7825" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7826">
+      <c r="A7826" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7826" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7827">
+      <c r="A7827" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7827" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7828">
+      <c r="A7828" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7828" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7829">
+      <c r="A7829" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7829" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7830">
+      <c r="A7830" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7830" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7831">
+      <c r="A7831" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7831" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7832">
+      <c r="A7832" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7832" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7833">
+      <c r="A7833" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7833" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7834">
+      <c r="A7834" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7834" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7835">
+      <c r="A7835" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7835" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7836">
+      <c r="A7836" t="n">
+        <v>23</v>
+      </c>
+      <c r="B7836" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7837">
+      <c r="A7837" t="n">
+        <v>23</v>
+      </c>
+      <c r="B7837" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7838">
+      <c r="A7838" t="n">
+        <v>23</v>
+      </c>
+      <c r="B7838" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7839">
+      <c r="A7839" t="n">
+        <v>23.33333333333333</v>
+      </c>
+      <c r="B7839" t="n">
+        <v>23.33333333333333</v>
+      </c>
+    </row>
+    <row r="7840">
+      <c r="A7840" t="n">
+        <v>23.33333333333333</v>
+      </c>
+      <c r="B7840" t="n">
+        <v>23.33333333333333</v>
+      </c>
+    </row>
+    <row r="7841">
+      <c r="A7841" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="B7841" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="7842">
+      <c r="A7842" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="B7842" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="7843">
+      <c r="A7843" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="B7843" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="7844">
+      <c r="A7844" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="B7844" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="7845">
+      <c r="A7845" t="n">
+        <v>24.14285714285714</v>
+      </c>
+      <c r="B7845" t="n">
+        <v>24.14285714285714</v>
+      </c>
+    </row>
+    <row r="7846">
+      <c r="A7846" t="n">
+        <v>24.14285714285714</v>
+      </c>
+      <c r="B7846" t="n">
+        <v>24.14285714285714</v>
+      </c>
+    </row>
+    <row r="7847">
+      <c r="A7847" t="n">
+        <v>24.14285714285714</v>
+      </c>
+      <c r="B7847" t="n">
+        <v>24.14285714285714</v>
+      </c>
+    </row>
+    <row r="7848">
+      <c r="A7848" t="n">
+        <v>24.44444444444444</v>
+      </c>
+      <c r="B7848" t="n">
+        <v>24.44444444444444</v>
+      </c>
+    </row>
+    <row r="7849">
+      <c r="A7849" t="n">
+        <v>24.44444444444444</v>
+      </c>
+      <c r="B7849" t="n">
+        <v>24.44444444444444</v>
+      </c>
+    </row>
+    <row r="7850">
+      <c r="A7850" t="n">
+        <v>24.44444444444444</v>
+      </c>
+      <c r="B7850" t="n">
+        <v>24.44444444444444</v>
+      </c>
+    </row>
+    <row r="7851">
+      <c r="A7851" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="B7851" t="n">
+        <v>24.6</v>
+      </c>
+    </row>
+    <row r="7852">
+      <c r="A7852" t="n">
+        <v>24.72727272727273</v>
+      </c>
+      <c r="B7852" t="n">
+        <v>24.72727272727273</v>
+      </c>
+    </row>
+    <row r="7853">
+      <c r="A7853" t="n">
+        <v>24.72727272727273</v>
+      </c>
+      <c r="B7853" t="n">
+        <v>24.72727272727273</v>
+      </c>
+    </row>
+    <row r="7854">
+      <c r="A7854" t="n">
+        <v>25.30769230769231</v>
+      </c>
+      <c r="B7854" t="n">
+        <v>25.30769230769231</v>
+      </c>
+    </row>
+    <row r="7855">
+      <c r="A7855" t="n">
+        <v>25.30769230769231</v>
+      </c>
+      <c r="B7855" t="n">
+        <v>25.30769230769231</v>
+      </c>
+    </row>
+    <row r="7856">
+      <c r="A7856" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="B7856" t="n">
+        <v>25.42857142857143</v>
+      </c>
+    </row>
+    <row r="7857">
+      <c r="A7857" t="n">
+        <v>25.53333333333333</v>
+      </c>
+      <c r="B7857" t="n">
+        <v>25.53333333333333</v>
+      </c>
+    </row>
+    <row r="7858">
+      <c r="A7858" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B7858" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="7859">
+      <c r="A7859" t="n">
+        <v>25.77777777777778</v>
+      </c>
+      <c r="B7859" t="n">
+        <v>25.77777777777778</v>
+      </c>
+    </row>
+    <row r="7860">
+      <c r="A7860" t="n">
+        <v>25.84210526315789</v>
+      </c>
+      <c r="B7860" t="n">
+        <v>25.84210526315789</v>
+      </c>
+    </row>
+    <row r="7861">
+      <c r="A7861" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="B7861" t="n">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="7862">
+      <c r="A7862" t="n">
+        <v>25.76190476190476</v>
+      </c>
+      <c r="B7862" t="n">
+        <v>25.76190476190476</v>
+      </c>
+    </row>
+    <row r="7863">
+      <c r="A7863" t="n">
+        <v>25.77272727272727</v>
+      </c>
+      <c r="B7863" t="n">
+        <v>25.77272727272727</v>
+      </c>
+    </row>
+    <row r="7864">
+      <c r="A7864" t="n">
+        <v>25.73913043478261</v>
+      </c>
+      <c r="B7864" t="n">
+        <v>25.73913043478261</v>
+      </c>
+    </row>
+    <row r="7865">
+      <c r="A7865" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="B7865" t="n">
+        <v>25.64</v>
+      </c>
+    </row>
+    <row r="7866">
+      <c r="A7866" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="B7866" t="n">
+        <v>25.64</v>
+      </c>
+    </row>
+    <row r="7867">
+      <c r="A7867" t="n">
+        <v>25.44444444444444</v>
+      </c>
+      <c r="B7867" t="n">
+        <v>25.44444444444444</v>
+      </c>
+    </row>
+    <row r="7868">
+      <c r="A7868" t="n">
+        <v>25.44444444444444</v>
+      </c>
+      <c r="B7868" t="n">
+        <v>25.44444444444444</v>
+      </c>
+    </row>
+    <row r="7869">
+      <c r="A7869" t="n">
+        <v>25.39285714285714</v>
+      </c>
+      <c r="B7869" t="n">
+        <v>25.39285714285714</v>
+      </c>
+    </row>
+    <row r="7870">
+      <c r="A7870" t="n">
+        <v>25.39285714285714</v>
+      </c>
+      <c r="B7870" t="n">
+        <v>25.39285714285714</v>
+      </c>
+    </row>
+    <row r="7871">
+      <c r="A7871" t="n">
+        <v>25.39285714285714</v>
+      </c>
+      <c r="B7871" t="n">
+        <v>25.39285714285714</v>
+      </c>
+    </row>
+    <row r="7872">
+      <c r="A7872" t="n">
+        <v>25.39285714285714</v>
+      </c>
+      <c r="B7872" t="n">
+        <v>25.39285714285714</v>
+      </c>
+    </row>
+    <row r="7873">
+      <c r="A7873" t="n">
+        <v>25.44827586206896</v>
+      </c>
+      <c r="B7873" t="n">
+        <v>25.44827586206896</v>
+      </c>
+    </row>
+    <row r="7874">
+      <c r="A7874" t="n">
+        <v>25.44827586206896</v>
+      </c>
+      <c r="B7874" t="n">
+        <v>25.44827586206896</v>
+      </c>
+    </row>
+    <row r="7875">
+      <c r="A7875" t="n">
+        <v>25.54838709677419</v>
+      </c>
+      <c r="B7875" t="n">
+        <v>25.54838709677419</v>
+      </c>
+    </row>
+    <row r="7876">
+      <c r="A7876" t="n">
+        <v>25.5625</v>
+      </c>
+      <c r="B7876" t="n">
+        <v>25.5625</v>
+      </c>
+    </row>
+    <row r="7877">
+      <c r="A7877" t="n">
+        <v>25.54545454545455</v>
+      </c>
+      <c r="B7877" t="n">
+        <v>25.54545454545455</v>
+      </c>
+    </row>
+    <row r="7878">
+      <c r="A7878" t="n">
+        <v>25.64705882352941</v>
+      </c>
+      <c r="B7878" t="n">
+        <v>25.64705882352941</v>
+      </c>
+    </row>
+    <row r="7879">
+      <c r="A7879" t="n">
+        <v>25.64705882352941</v>
+      </c>
+      <c r="B7879" t="n">
+        <v>25.64705882352941</v>
+      </c>
+    </row>
+    <row r="7880">
+      <c r="A7880" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="B7880" t="n">
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="7881">
+      <c r="A7881" t="n">
+        <v>25.64864864864865</v>
+      </c>
+      <c r="B7881" t="n">
+        <v>25.64864864864865</v>
+      </c>
+    </row>
+    <row r="7882">
+      <c r="A7882" t="n">
+        <v>25.60526315789474</v>
+      </c>
+      <c r="B7882" t="n">
+        <v>25.60526315789474</v>
+      </c>
+    </row>
+    <row r="7883">
+      <c r="A7883" t="n">
+        <v>25.60526315789474</v>
+      </c>
+      <c r="B7883" t="n">
+        <v>25.60526315789474</v>
+      </c>
+    </row>
+    <row r="7884">
+      <c r="A7884" t="n">
+        <v>25.53846153846154</v>
+      </c>
+      <c r="B7884" t="n">
+        <v>25.53846153846154</v>
+      </c>
+    </row>
+    <row r="7885">
+      <c r="A7885" t="n">
+        <v>25.53846153846154</v>
+      </c>
+      <c r="B7885" t="n">
+        <v>25.53846153846154</v>
+      </c>
+    </row>
+    <row r="7886">
+      <c r="A7886" t="n">
+        <v>25.53846153846154</v>
+      </c>
+      <c r="B7886" t="n">
+        <v>25.53846153846154</v>
+      </c>
+    </row>
+    <row r="7887">
+      <c r="A7887" t="n">
+        <v>25.53846153846154</v>
+      </c>
+      <c r="B7887" t="n">
+        <v>25.53846153846154</v>
+      </c>
+    </row>
+    <row r="7888">
+      <c r="A7888" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B7888" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="7889">
+      <c r="A7889" t="n">
+        <v>25.48780487804878</v>
+      </c>
+      <c r="B7889" t="n">
+        <v>25.48780487804878</v>
+      </c>
+    </row>
+    <row r="7890">
+      <c r="A7890" t="n">
+        <v>25.46511627906977</v>
+      </c>
+      <c r="B7890" t="n">
+        <v>25.46511627906977</v>
+      </c>
+    </row>
+    <row r="7891">
+      <c r="A7891" t="n">
+        <v>25.46511627906977</v>
+      </c>
+      <c r="B7891" t="n">
+        <v>25.46511627906977</v>
+      </c>
+    </row>
+    <row r="7892">
+      <c r="A7892" t="n">
+        <v>25.35555555555555</v>
+      </c>
+      <c r="B7892" t="n">
+        <v>25.35555555555555</v>
+      </c>
+    </row>
+    <row r="7893">
+      <c r="A7893" t="n">
+        <v>25.35555555555555</v>
+      </c>
+      <c r="B7893" t="n">
+        <v>25.35555555555555</v>
+      </c>
+    </row>
+    <row r="7894">
+      <c r="A7894" t="n">
+        <v>25.35555555555555</v>
+      </c>
+      <c r="B7894" t="n">
+        <v>25.35555555555555</v>
+      </c>
+    </row>
+    <row r="7895">
+      <c r="A7895" t="n">
+        <v>25.35555555555555</v>
+      </c>
+      <c r="B7895" t="n">
+        <v>25.35555555555555</v>
+      </c>
+    </row>
+    <row r="7896">
+      <c r="A7896" t="n">
+        <v>25.40909090909091</v>
+      </c>
+      <c r="B7896" t="n">
+        <v>25.35555555555555</v>
+      </c>
+    </row>
+    <row r="7897">
+      <c r="A7897" t="n">
+        <v>25.48888888888889</v>
+      </c>
+      <c r="B7897" t="n">
+        <v>25.38297872340426</v>
+      </c>
+    </row>
+    <row r="7898">
+      <c r="A7898" t="n">
+        <v>25.48888888888889</v>
+      </c>
+      <c r="B7898" t="n">
+        <v>25.38297872340426</v>
+      </c>
+    </row>
+    <row r="7899">
+      <c r="A7899" t="n">
+        <v>25.45652173913043</v>
+      </c>
+      <c r="B7899" t="n">
+        <v>25.3265306122449</v>
+      </c>
+    </row>
+    <row r="7900">
+      <c r="A7900" t="n">
+        <v>25.48936170212766</v>
+      </c>
+      <c r="B7900" t="n">
+        <v>25.36</v>
+      </c>
+    </row>
+    <row r="7901">
+      <c r="A7901" t="n">
+        <v>25.48936170212766</v>
+      </c>
+      <c r="B7901" t="n">
+        <v>25.33333333333333</v>
+      </c>
+    </row>
+    <row r="7902">
+      <c r="A7902" t="n">
+        <v>25.48936170212766</v>
+      </c>
+      <c r="B7902" t="n">
+        <v>25.33333333333333</v>
+      </c>
+    </row>
+    <row r="7903">
+      <c r="A7903" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B7903" t="n">
+        <v>25.33333333333333</v>
+      </c>
+    </row>
+    <row r="7904">
+      <c r="A7904" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B7904" t="n">
+        <v>25.33333333333333</v>
+      </c>
+    </row>
+    <row r="7905">
+      <c r="A7905" t="n">
+        <v>25.53191489361702</v>
+      </c>
+      <c r="B7905" t="n">
+        <v>25.35185185185185</v>
+      </c>
+    </row>
+    <row r="7906">
+      <c r="A7906" t="n">
+        <v>25.53191489361702</v>
+      </c>
+      <c r="B7906" t="n">
+        <v>25.35185185185185</v>
+      </c>
+    </row>
+    <row r="7907">
+      <c r="A7907" t="n">
+        <v>25.53191489361702</v>
+      </c>
+      <c r="B7907" t="n">
+        <v>25.35185185185185</v>
+      </c>
+    </row>
+    <row r="7908">
+      <c r="A7908" t="n">
+        <v>25.53333333333333</v>
+      </c>
+      <c r="B7908" t="n">
+        <v>25.35185185185185</v>
+      </c>
+    </row>
+    <row r="7909">
+      <c r="A7909" t="n">
+        <v>25.59574468085106</v>
+      </c>
+      <c r="B7909" t="n">
+        <v>25.41071428571428</v>
+      </c>
+    </row>
+    <row r="7910">
+      <c r="A7910" t="n">
+        <v>25.59574468085106</v>
+      </c>
+      <c r="B7910" t="n">
+        <v>25.41071428571428</v>
+      </c>
+    </row>
+    <row r="7911">
+      <c r="A7911" t="n">
+        <v>25.59574468085106</v>
+      </c>
+      <c r="B7911" t="n">
+        <v>25.42105263157895</v>
+      </c>
+    </row>
+    <row r="7912">
+      <c r="A7912" t="n">
+        <v>25.58695652173913</v>
+      </c>
+      <c r="B7912" t="n">
+        <v>25.42105263157895</v>
+      </c>
+    </row>
+    <row r="7913">
+      <c r="A7913" t="n">
+        <v>25.61702127659574</v>
+      </c>
+      <c r="B7913" t="n">
+        <v>25.44827586206896</v>
+      </c>
+    </row>
+    <row r="7914">
+      <c r="A7914" t="n">
+        <v>25.47826086956522</v>
+      </c>
+      <c r="B7914" t="n">
+        <v>25.4406779661017</v>
+      </c>
+    </row>
+    <row r="7915">
+      <c r="A7915" t="n">
+        <v>25.47826086956522</v>
+      </c>
+      <c r="B7915" t="n">
+        <v>25.4406779661017</v>
+      </c>
+    </row>
+    <row r="7916">
+      <c r="A7916" t="n">
+        <v>25.53191489361702</v>
+      </c>
+      <c r="B7916" t="n">
+        <v>25.50819672131147</v>
+      </c>
+    </row>
+    <row r="7917">
+      <c r="A7917" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B7917" t="n">
+        <v>25.50819672131147</v>
+      </c>
+    </row>
+    <row r="7918">
+      <c r="A7918" t="n">
+        <v>25.52173913043478</v>
+      </c>
+      <c r="B7918" t="n">
+        <v>25.51612903225806</v>
+      </c>
+    </row>
+    <row r="7919">
+      <c r="A7919" t="n">
+        <v>25.68085106382979</v>
+      </c>
+      <c r="B7919" t="n">
+        <v>25.70769230769231</v>
+      </c>
+    </row>
+    <row r="7920">
+      <c r="A7920" t="n">
+        <v>25.65217391304348</v>
+      </c>
+      <c r="B7920" t="n">
+        <v>25.70769230769231</v>
+      </c>
+    </row>
+    <row r="7921">
+      <c r="A7921" t="n">
+        <v>25.6875</v>
+      </c>
+      <c r="B7921" t="n">
+        <v>25.72058823529412</v>
+      </c>
+    </row>
+    <row r="7922">
+      <c r="A7922" t="n">
+        <v>25.70212765957447</v>
+      </c>
+      <c r="B7922" t="n">
+        <v>25.72058823529412</v>
+      </c>
+    </row>
+    <row r="7923">
+      <c r="A7923" t="n">
+        <v>25.6530612244898</v>
+      </c>
+      <c r="B7923" t="n">
+        <v>25.69014084507042</v>
+      </c>
+    </row>
+    <row r="7924">
+      <c r="A7924" t="n">
+        <v>25.66666666666667</v>
+      </c>
+      <c r="B7924" t="n">
+        <v>25.69014084507042</v>
+      </c>
+    </row>
+    <row r="7925">
+      <c r="A7925" t="n">
+        <v>25.68085106382979</v>
+      </c>
+      <c r="B7925" t="n">
+        <v>25.66666666666667</v>
+      </c>
+    </row>
+    <row r="7926">
+      <c r="A7926" t="n">
+        <v>25.68085106382979</v>
+      </c>
+      <c r="B7926" t="n">
+        <v>25.66666666666667</v>
+      </c>
+    </row>
+    <row r="7927">
+      <c r="A7927" t="n">
+        <v>25.78260869565218</v>
+      </c>
+      <c r="B7927" t="n">
+        <v>25.65753424657534</v>
+      </c>
+    </row>
+    <row r="7928">
+      <c r="A7928" t="n">
+        <v>25.78260869565218</v>
+      </c>
+      <c r="B7928" t="n">
+        <v>25.65753424657534</v>
+      </c>
+    </row>
+    <row r="7929">
+      <c r="A7929" t="n">
+        <v>25.91304347826087</v>
+      </c>
+      <c r="B7929" t="n">
+        <v>25.71621621621622</v>
+      </c>
+    </row>
+    <row r="7930">
+      <c r="A7930" t="n">
+        <v>25.91304347826087</v>
+      </c>
+      <c r="B7930" t="n">
+        <v>25.71621621621622</v>
+      </c>
+    </row>
+    <row r="7931">
+      <c r="A7931" t="n">
+        <v>25.8936170212766</v>
+      </c>
+      <c r="B7931" t="n">
+        <v>25.70666666666667</v>
+      </c>
+    </row>
+    <row r="7932">
+      <c r="A7932" t="n">
+        <v>25.91666666666667</v>
+      </c>
+      <c r="B7932" t="n">
+        <v>25.72368421052632</v>
+      </c>
+    </row>
+    <row r="7933">
+      <c r="A7933" t="n">
+        <v>25.875</v>
+      </c>
+      <c r="B7933" t="n">
+        <v>25.71428571428572</v>
+      </c>
+    </row>
+    <row r="7934">
+      <c r="A7934" t="n">
+        <v>25.875</v>
+      </c>
+      <c r="B7934" t="n">
+        <v>25.71428571428572</v>
+      </c>
+    </row>
+    <row r="7935">
+      <c r="A7935" t="n">
+        <v>25.82978723404255</v>
+      </c>
+      <c r="B7935" t="n">
+        <v>25.71794871794872</v>
+      </c>
+    </row>
+    <row r="7936">
+      <c r="A7936" t="n">
+        <v>25.82608695652174</v>
+      </c>
+      <c r="B7936" t="n">
+        <v>25.71794871794872</v>
+      </c>
+    </row>
+    <row r="7937">
+      <c r="A7937" t="n">
+        <v>26.04255319148936</v>
+      </c>
+      <c r="B7937" t="n">
+        <v>25.8375</v>
+      </c>
+    </row>
+    <row r="7938">
+      <c r="A7938" t="n">
+        <v>25.97826086956522</v>
+      </c>
+      <c r="B7938" t="n">
+        <v>25.8375</v>
+      </c>
+    </row>
+    <row r="7939">
+      <c r="A7939" t="n">
+        <v>26</v>
+      </c>
+      <c r="B7939" t="n">
+        <v>25.85365853658537</v>
+      </c>
+    </row>
+    <row r="7940">
+      <c r="A7940" t="n">
+        <v>26.29166666666667</v>
+      </c>
+      <c r="B7940" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7941">
+      <c r="A7941" t="n">
+        <v>26.21276595744681</v>
+      </c>
+      <c r="B7941" t="n">
+        <v>25.96428571428572</v>
+      </c>
+    </row>
+    <row r="7942">
+      <c r="A7942" t="n">
+        <v>26.23404255319149</v>
+      </c>
+      <c r="B7942" t="n">
+        <v>25.95294117647059</v>
+      </c>
+    </row>
+    <row r="7943">
+      <c r="A7943" t="n">
+        <v>26.23404255319149</v>
+      </c>
+      <c r="B7943" t="n">
+        <v>25.95294117647059</v>
+      </c>
+    </row>
+    <row r="7944">
+      <c r="A7944" t="n">
+        <v>26.30434782608696</v>
+      </c>
+      <c r="B7944" t="n">
+        <v>25.95294117647059</v>
+      </c>
+    </row>
+    <row r="7945">
+      <c r="A7945" t="n">
+        <v>26.30434782608696</v>
+      </c>
+      <c r="B7945" t="n">
+        <v>25.95294117647059</v>
+      </c>
+    </row>
+    <row r="7946">
+      <c r="A7946" t="n">
+        <v>26.27659574468085</v>
+      </c>
+      <c r="B7946" t="n">
+        <v>25.94186046511628</v>
+      </c>
+    </row>
+    <row r="7947">
+      <c r="A7947" t="n">
+        <v>26.27659574468085</v>
+      </c>
+      <c r="B7947" t="n">
+        <v>25.94186046511628</v>
+      </c>
+    </row>
+    <row r="7948">
+      <c r="A7948" t="n">
+        <v>26.32608695652174</v>
+      </c>
+      <c r="B7948" t="n">
+        <v>25.94186046511628</v>
+      </c>
+    </row>
+    <row r="7949">
+      <c r="A7949" t="n">
+        <v>26.35555555555555</v>
+      </c>
+      <c r="B7949" t="n">
+        <v>25.94186046511628</v>
+      </c>
+    </row>
+    <row r="7950">
+      <c r="A7950" t="n">
+        <v>26.41860465116279</v>
+      </c>
+      <c r="B7950" t="n">
+        <v>25.94186046511628</v>
+      </c>
+    </row>
+    <row r="7951">
+      <c r="A7951" t="n">
+        <v>26.45454545454545</v>
+      </c>
+      <c r="B7951" t="n">
+        <v>25.96551724137931</v>
+      </c>
+    </row>
+    <row r="7952">
+      <c r="A7952" t="n">
+        <v>26.55813953488372</v>
+      </c>
+      <c r="B7952" t="n">
+        <v>25.94318181818182</v>
+      </c>
+    </row>
+    <row r="7953">
+      <c r="A7953" t="n">
+        <v>26.61363636363636</v>
+      </c>
+      <c r="B7953" t="n">
+        <v>25.97752808988764</v>
+      </c>
+    </row>
+    <row r="7954">
+      <c r="A7954" t="n">
+        <v>26.61363636363636</v>
+      </c>
+      <c r="B7954" t="n">
+        <v>25.97752808988764</v>
+      </c>
+    </row>
+    <row r="7955">
+      <c r="A7955" t="n">
+        <v>26.55555555555556</v>
+      </c>
+      <c r="B7955" t="n">
+        <v>25.95555555555556</v>
+      </c>
+    </row>
+    <row r="7956">
+      <c r="A7956" t="n">
+        <v>26.55555555555556</v>
+      </c>
+      <c r="B7956" t="n">
+        <v>25.95555555555556</v>
+      </c>
+    </row>
+    <row r="7957">
+      <c r="A7957" t="n">
+        <v>26.58139534883721</v>
+      </c>
+      <c r="B7957" t="n">
+        <v>25.95555555555556</v>
+      </c>
+    </row>
+    <row r="7958">
+      <c r="A7958" t="n">
+        <v>26.61363636363636</v>
+      </c>
+      <c r="B7958" t="n">
+        <v>25.97802197802198</v>
+      </c>
+    </row>
+    <row r="7959">
+      <c r="A7959" t="n">
+        <v>26.73809523809524</v>
+      </c>
+      <c r="B7959" t="n">
+        <v>25.97802197802198</v>
+      </c>
+    </row>
+    <row r="7960">
+      <c r="A7960" t="n">
+        <v>26.71428571428572</v>
+      </c>
+      <c r="B7960" t="n">
+        <v>25.97826086956522</v>
+      </c>
+    </row>
+    <row r="7961">
+      <c r="A7961" t="n">
+        <v>26.78048780487805</v>
+      </c>
+      <c r="B7961" t="n">
+        <v>25.97826086956522</v>
+      </c>
+    </row>
+    <row r="7962">
+      <c r="A7962" t="n">
+        <v>26.73809523809524</v>
+      </c>
+      <c r="B7962" t="n">
+        <v>25.96774193548387</v>
+      </c>
+    </row>
+    <row r="7963">
+      <c r="A7963" t="n">
+        <v>26.73809523809524</v>
+      </c>
+      <c r="B7963" t="n">
+        <v>25.96774193548387</v>
+      </c>
+    </row>
+    <row r="7964">
+      <c r="A7964" t="n">
+        <v>26.73809523809524</v>
+      </c>
+      <c r="B7964" t="n">
+        <v>25.96774193548387</v>
+      </c>
+    </row>
+    <row r="7965">
+      <c r="A7965" t="n">
+        <v>26.82051282051282</v>
+      </c>
+      <c r="B7965" t="n">
+        <v>25.96774193548387</v>
+      </c>
+    </row>
+    <row r="7966">
+      <c r="A7966" t="n">
+        <v>26.82051282051282</v>
+      </c>
+      <c r="B7966" t="n">
+        <v>25.96774193548387</v>
+      </c>
+    </row>
+    <row r="7967">
+      <c r="A7967" t="n">
+        <v>26.825</v>
+      </c>
+      <c r="B7967" t="n">
+        <v>25.97872340425532</v>
+      </c>
+    </row>
+    <row r="7968">
+      <c r="A7968" t="n">
+        <v>26.825</v>
+      </c>
+      <c r="B7968" t="n">
+        <v>25.97872340425532</v>
+      </c>
+    </row>
+    <row r="7969">
+      <c r="A7969" t="n">
+        <v>26.95</v>
+      </c>
+      <c r="B7969" t="n">
+        <v>26.05208333333333</v>
+      </c>
+    </row>
+    <row r="7970">
+      <c r="A7970" t="n">
+        <v>26.95</v>
+      </c>
+      <c r="B7970" t="n">
+        <v>26.05208333333333</v>
+      </c>
+    </row>
+    <row r="7971">
+      <c r="A7971" t="n">
+        <v>26.925</v>
+      </c>
+      <c r="B7971" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7972">
+      <c r="A7972" t="n">
+        <v>26.925</v>
+      </c>
+      <c r="B7972" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7973">
+      <c r="A7973" t="n">
+        <v>26.92307692307692</v>
+      </c>
+      <c r="B7973" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7974">
+      <c r="A7974" t="n">
+        <v>26.97368421052632</v>
+      </c>
+      <c r="B7974" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7975">
+      <c r="A7975" t="n">
+        <v>26.97368421052632</v>
+      </c>
+      <c r="B7975" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7976">
+      <c r="A7976" t="n">
+        <v>26.94444444444444</v>
+      </c>
+      <c r="B7976" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7977">
+      <c r="A7977" t="n">
+        <v>26.94444444444444</v>
+      </c>
+      <c r="B7977" t="n">
+        <v>26.04123711340206</v>
+      </c>
+    </row>
+    <row r="7978">
+      <c r="A7978" t="n">
+        <v>27</v>
+      </c>
+      <c r="B7978" t="n">
+        <v>26.06122448979592</v>
+      </c>
+    </row>
+    <row r="7979">
+      <c r="A7979" t="n">
+        <v>26.73529411764706</v>
+      </c>
+      <c r="B7979" t="n">
+        <v>26.06060606060606</v>
+      </c>
+    </row>
+    <row r="7980">
+      <c r="A7980" t="n">
+        <v>26.75</v>
+      </c>
+      <c r="B7980" t="n">
+        <v>26.07920792079208</v>
+      </c>
+    </row>
+    <row r="7981">
+      <c r="A7981" t="n">
+        <v>26.81818181818182</v>
+      </c>
+      <c r="B7981" t="n">
+        <v>26.07920792079208</v>
+      </c>
+    </row>
+    <row r="7982">
+      <c r="A7982" t="n">
+        <v>26.79411764705882</v>
+      </c>
+      <c r="B7982" t="n">
+        <v>26.07843137254902</v>
+      </c>
+    </row>
+    <row r="7983">
+      <c r="A7983" t="n">
+        <v>26.96774193548387</v>
+      </c>
+      <c r="B7983" t="n">
+        <v>26.07843137254902</v>
+      </c>
+    </row>
+    <row r="7984">
+      <c r="A7984" t="n">
+        <v>26.96774193548387</v>
+      </c>
+      <c r="B7984" t="n">
+        <v>26.07843137254902</v>
+      </c>
+    </row>
+    <row r="7985">
+      <c r="A7985" t="n">
+        <v>27.06666666666667</v>
+      </c>
+      <c r="B7985" t="n">
+        <v>26.07843137254902</v>
+      </c>
+    </row>
+    <row r="7986">
+      <c r="A7986" t="n">
+        <v>27.03225806451613</v>
+      </c>
+      <c r="B7986" t="n">
+        <v>26.07766990291262</v>
+      </c>
+    </row>
+    <row r="7987">
+      <c r="A7987" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="B7987" t="n">
+        <v>26.07766990291262</v>
+      </c>
+    </row>
+    <row r="7988">
+      <c r="A7988" t="n">
+        <v>27.03225806451613</v>
+      </c>
+      <c r="B7988" t="n">
+        <v>26.06730769230769</v>
+      </c>
+    </row>
+    <row r="7989">
+      <c r="A7989" t="n">
+        <v>26.93333333333333</v>
+      </c>
+      <c r="B7989" t="n">
+        <v>26.06730769230769</v>
+      </c>
+    </row>
+    <row r="7990">
+      <c r="A7990" t="n">
+        <v>26.90322580645161</v>
+      </c>
+      <c r="B7990" t="n">
+        <v>26.06666666666667</v>
+      </c>
+    </row>
+    <row r="7991">
+      <c r="A7991" t="n">
+        <v>26.87096774193548</v>
+      </c>
+      <c r="B7991" t="n">
+        <v>26.04716981132075</v>
+      </c>
+    </row>
+    <row r="7992">
+      <c r="A7992" t="n">
+        <v>26.86666666666667</v>
+      </c>
+      <c r="B7992" t="n">
+        <v>26.04716981132075</v>
+      </c>
+    </row>
+    <row r="7993">
+      <c r="A7993" t="n">
+        <v>26.93103448275862</v>
+      </c>
+      <c r="B7993" t="n">
+        <v>26.04716981132075</v>
+      </c>
+    </row>
+    <row r="7994">
+      <c r="A7994" t="n">
+        <v>26.93103448275862</v>
+      </c>
+      <c r="B7994" t="n">
+        <v>26.04716981132075</v>
+      </c>
+    </row>
+    <row r="7995">
+      <c r="A7995" t="n">
+        <v>26.86206896551724</v>
+      </c>
+      <c r="B7995" t="n">
+        <v>26.02803738317757</v>
+      </c>
+    </row>
+    <row r="7996">
+      <c r="A7996" t="n">
+        <v>26.83333333333333</v>
+      </c>
+      <c r="B7996" t="n">
+        <v>26.02777777777778</v>
+      </c>
+    </row>
+    <row r="7997">
+      <c r="A7997" t="n">
+        <v>26.57142857142857</v>
+      </c>
+      <c r="B7997" t="n">
+        <v>26.02777777777778</v>
+      </c>
+    </row>
+    <row r="7998">
+      <c r="A7998" t="n">
+        <v>26.57142857142857</v>
+      </c>
+      <c r="B7998" t="n">
+        <v>26.02777777777778</v>
+      </c>
+    </row>
+    <row r="7999">
+      <c r="A7999" t="n">
+        <v>26.57692307692308</v>
+      </c>
+      <c r="B7999" t="n">
+        <v>26.02777777777778</v>
+      </c>
+    </row>
+    <row r="8000">
+      <c r="A8000" t="n">
+        <v>26.12</v>
+      </c>
+      <c r="B8000" t="n">
+        <v>26.02777777777778</v>
+      </c>
+    </row>
+    <row r="8001">
+      <c r="A8001" t="n">
+        <v>26.24</v>
+      </c>
+      <c r="B8001" t="n">
+        <v>26.02752293577982</v>
+      </c>
+    </row>
+    <row r="8002">
+      <c r="A8002" t="n">
+        <v>26.29166666666667</v>
+      </c>
+      <c r="B8002" t="n">
+        <v>26.02752293577982</v>
+      </c>
+    </row>
+    <row r="8003">
+      <c r="A8003" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="B8003" t="n">
+        <v>26.00909090909091</v>
+      </c>
+    </row>
+    <row r="8004">
+      <c r="A8004" t="n">
+        <v>26.23076923076923</v>
+      </c>
+      <c r="B8004" t="n">
+        <v>26.01801801801802</v>
+      </c>
+    </row>
+    <row r="8005">
+      <c r="A8005" t="n">
+        <v>26.23076923076923</v>
+      </c>
+      <c r="B8005" t="n">
+        <v>26.01801801801802</v>
+      </c>
+    </row>
+    <row r="8006">
+      <c r="A8006" t="n">
+        <v>26.19230769230769</v>
+      </c>
+      <c r="B8006" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8007">
+      <c r="A8007" t="n">
+        <v>26.19230769230769</v>
+      </c>
+      <c r="B8007" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8008">
+      <c r="A8008" t="n">
+        <v>26.19230769230769</v>
+      </c>
+      <c r="B8008" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8009">
+      <c r="A8009" t="n">
+        <v>26.14814814814815</v>
+      </c>
+      <c r="B8009" t="n">
+        <v>25.99115044247788</v>
+      </c>
+    </row>
+    <row r="8010">
+      <c r="A8010" t="n">
+        <v>26.17857142857143</v>
+      </c>
+      <c r="B8010" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8011">
+      <c r="A8011" t="n">
+        <v>26.11111111111111</v>
+      </c>
+      <c r="B8011" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8012">
+      <c r="A8012" t="n">
+        <v>26.14814814814815</v>
+      </c>
+      <c r="B8012" t="n">
+        <v>25.99130434782609</v>
+      </c>
+    </row>
+    <row r="8013">
+      <c r="A8013" t="n">
+        <v>26.03846153846154</v>
+      </c>
+      <c r="B8013" t="n">
+        <v>25.99130434782609</v>
+      </c>
+    </row>
+    <row r="8014">
+      <c r="A8014" t="n">
+        <v>26.03571428571428</v>
+      </c>
+      <c r="B8014" t="n">
+        <v>25.99145299145299</v>
+      </c>
+    </row>
+    <row r="8015">
+      <c r="A8015" t="n">
+        <v>26.11111111111111</v>
+      </c>
+      <c r="B8015" t="n">
+        <v>25.99145299145299</v>
+      </c>
+    </row>
+    <row r="8016">
+      <c r="A8016" t="n">
+        <v>26.11111111111111</v>
+      </c>
+      <c r="B8016" t="n">
+        <v>25.99145299145299</v>
+      </c>
+    </row>
+    <row r="8017">
+      <c r="A8017" t="n">
+        <v>26.11111111111111</v>
+      </c>
+      <c r="B8017" t="n">
+        <v>25.99145299145299</v>
+      </c>
+    </row>
+    <row r="8018">
+      <c r="A8018" t="n">
+        <v>26.03846153846154</v>
+      </c>
+      <c r="B8018" t="n">
+        <v>25.99145299145299</v>
+      </c>
+    </row>
+    <row r="8019">
+      <c r="A8019" t="n">
+        <v>26.07142857142857</v>
+      </c>
+      <c r="B8019" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8020">
+      <c r="A8020" t="n">
+        <v>26.07407407407407</v>
+      </c>
+      <c r="B8020" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8021">
+      <c r="A8021" t="n">
+        <v>26.21428571428572</v>
+      </c>
+      <c r="B8021" t="n">
+        <v>26.03333333333333</v>
+      </c>
+    </row>
+    <row r="8022">
+      <c r="A8022" t="n">
+        <v>26.10344827586207</v>
+      </c>
+      <c r="B8022" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8023">
+      <c r="A8023" t="n">
+        <v>26.10344827586207</v>
+      </c>
+      <c r="B8023" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8024">
+      <c r="A8024" t="n">
+        <v>26</v>
+      </c>
+      <c r="B8024" t="n">
+        <v>25.97560975609756</v>
+      </c>
+    </row>
+    <row r="8025">
+      <c r="A8025" t="n">
+        <v>26</v>
+      </c>
+      <c r="B8025" t="n">
+        <v>25.97560975609756</v>
+      </c>
+    </row>
+    <row r="8026">
+      <c r="A8026" t="n">
+        <v>26</v>
+      </c>
+      <c r="B8026" t="n">
+        <v>25.97560975609756</v>
+      </c>
+    </row>
+    <row r="8027">
+      <c r="A8027" t="n">
+        <v>25.96666666666667</v>
+      </c>
+      <c r="B8027" t="n">
+        <v>25.9758064516129</v>
+      </c>
+    </row>
+    <row r="8028">
+      <c r="A8028" t="n">
+        <v>25.96666666666667</v>
+      </c>
+      <c r="B8028" t="n">
+        <v>25.9758064516129</v>
+      </c>
+    </row>
+    <row r="8029">
+      <c r="A8029" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B8029" t="n">
+        <v>25.9758064516129</v>
+      </c>
+    </row>
+    <row r="8030">
+      <c r="A8030" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B8030" t="n">
+        <v>25.9758064516129</v>
+      </c>
+    </row>
+    <row r="8031">
+      <c r="A8031" t="n">
+        <v>25.74074074074074</v>
+      </c>
+      <c r="B8031" t="n">
+        <v>25.9758064516129</v>
+      </c>
+    </row>
+    <row r="8032">
+      <c r="A8032" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="B8032" t="n">
+        <v>25.976</v>
+      </c>
+    </row>
+    <row r="8033">
+      <c r="A8033" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="B8033" t="n">
+        <v>25.93700787401575</v>
+      </c>
+    </row>
+    <row r="8034">
+      <c r="A8034" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="B8034" t="n">
+        <v>25.93700787401575</v>
+      </c>
+    </row>
+    <row r="8035">
+      <c r="A8035" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="B8035" t="n">
+        <v>25.93700787401575</v>
+      </c>
+    </row>
+    <row r="8036">
+      <c r="A8036" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="B8036" t="n">
+        <v>25.93700787401575</v>
+      </c>
+    </row>
+    <row r="8037">
+      <c r="A8037" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="B8037" t="n">
+        <v>25.93700787401575</v>
+      </c>
+    </row>
+    <row r="8038">
+      <c r="A8038" t="n">
+        <v>25.51724137931035</v>
+      </c>
+      <c r="B8038" t="n">
+        <v>25.93700787401575</v>
+      </c>
+    </row>
+    <row r="8039">
+      <c r="A8039" t="n">
+        <v>25.44827586206896</v>
+      </c>
+      <c r="B8039" t="n">
+        <v>25.921875</v>
+      </c>
+    </row>
+    <row r="8040">
+      <c r="A8040" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8040" t="n">
+        <v>25.921875</v>
+      </c>
+    </row>
+    <row r="8041">
+      <c r="A8041" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8041" t="n">
+        <v>25.921875</v>
+      </c>
+    </row>
+    <row r="8042">
+      <c r="A8042" t="n">
+        <v>25.30769230769231</v>
+      </c>
+      <c r="B8042" t="n">
+        <v>25.921875</v>
+      </c>
+    </row>
+    <row r="8043">
+      <c r="A8043" t="n">
+        <v>25.25925925925926</v>
+      </c>
+      <c r="B8043" t="n">
+        <v>25.90697674418605</v>
+      </c>
+    </row>
+    <row r="8044">
+      <c r="A8044" t="n">
+        <v>25.28571428571428</v>
+      </c>
+      <c r="B8044" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8045">
+      <c r="A8045" t="n">
+        <v>25.28571428571428</v>
+      </c>
+      <c r="B8045" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8046">
+      <c r="A8046" t="n">
+        <v>25.25925925925926</v>
+      </c>
+      <c r="B8046" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8047">
+      <c r="A8047" t="n">
+        <v>25.25925925925926</v>
+      </c>
+      <c r="B8047" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8048">
+      <c r="A8048" t="n">
+        <v>25.26923076923077</v>
+      </c>
+      <c r="B8048" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8049">
+      <c r="A8049" t="n">
+        <v>25.26923076923077</v>
+      </c>
+      <c r="B8049" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8050">
+      <c r="A8050" t="n">
+        <v>25.24</v>
+      </c>
+      <c r="B8050" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8051">
+      <c r="A8051" t="n">
+        <v>25.29166666666667</v>
+      </c>
+      <c r="B8051" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8052">
+      <c r="A8052" t="n">
+        <v>25.29166666666667</v>
+      </c>
+      <c r="B8052" t="n">
+        <v>25.90769230769231</v>
+      </c>
+    </row>
+    <row r="8053">
+      <c r="A8053" t="n">
+        <v>25.28</v>
+      </c>
+      <c r="B8053" t="n">
+        <v>25.90076335877863</v>
+      </c>
+    </row>
+    <row r="8054">
+      <c r="A8054" t="n">
+        <v>25.28</v>
+      </c>
+      <c r="B8054" t="n">
+        <v>25.90076335877863</v>
+      </c>
+    </row>
+    <row r="8055">
+      <c r="A8055" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8055" t="n">
+        <v>25.90076335877863</v>
+      </c>
+    </row>
+    <row r="8056">
+      <c r="A8056" t="n">
+        <v>25.30434782608696</v>
+      </c>
+      <c r="B8056" t="n">
+        <v>25.90076335877863</v>
+      </c>
+    </row>
+    <row r="8057">
+      <c r="A8057" t="n">
+        <v>25.30434782608696</v>
+      </c>
+      <c r="B8057" t="n">
+        <v>25.90076335877863</v>
+      </c>
+    </row>
+    <row r="8058">
+      <c r="A8058" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8058" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8059">
+      <c r="A8059" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8059" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8060">
+      <c r="A8060" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8060" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8061">
+      <c r="A8061" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8061" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8062">
+      <c r="A8062" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8062" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8063">
+      <c r="A8063" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8063" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8064">
+      <c r="A8064" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8064" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8065">
+      <c r="A8065" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8065" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8066">
+      <c r="A8066" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8066" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8067">
+      <c r="A8067" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8067" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8068">
+      <c r="A8068" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8068" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8069">
+      <c r="A8069" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8069" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8070">
+      <c r="A8070" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8070" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8071">
+      <c r="A8071" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8071" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8072">
+      <c r="A8072" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8072" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8073">
+      <c r="A8073" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8073" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8074">
+      <c r="A8074" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8074" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8075">
+      <c r="A8075" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8075" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8076">
+      <c r="A8076" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8076" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8077">
+      <c r="A8077" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8077" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8078">
+      <c r="A8078" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8078" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8079">
+      <c r="A8079" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8079" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8080">
+      <c r="A8080" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8080" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8081">
+      <c r="A8081" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8081" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8082">
+      <c r="A8082" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8082" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8083">
+      <c r="A8083" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8083" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8084">
+      <c r="A8084" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8084" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8085">
+      <c r="A8085" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8085" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8086">
+      <c r="A8086" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8086" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8087">
+      <c r="A8087" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8087" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8088">
+      <c r="A8088" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8088" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8089">
+      <c r="A8089" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8089" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8090">
+      <c r="A8090" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8090" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8091">
+      <c r="A8091" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8091" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8092">
+      <c r="A8092" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8092" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8093">
+      <c r="A8093" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8093" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8094">
+      <c r="A8094" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8094" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8095">
+      <c r="A8095" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8095" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8096">
+      <c r="A8096" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8096" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8097">
+      <c r="A8097" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8097" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8098">
+      <c r="A8098" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8098" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8099">
+      <c r="A8099" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8099" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8100">
+      <c r="A8100" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8101">
+      <c r="A8101" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8102">
+      <c r="A8102" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8103">
+      <c r="A8103" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8104">
+      <c r="A8104" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8104" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8105">
+      <c r="A8105" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8106">
+      <c r="A8106" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8107">
+      <c r="A8107" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8108">
+      <c r="A8108" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8109">
+      <c r="A8109" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8110">
+      <c r="A8110" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8111">
+      <c r="A8111" t="n">
+        <v>0</v>
+      </c>
+      <c r="B8111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8112">
+      <c r="A8112" t="n">
+        <v>23</v>
+      </c>
+      <c r="B8112" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8113">
+      <c r="A8113" t="n">
+        <v>23</v>
+      </c>
+      <c r="B8113" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8114">
+      <c r="A8114" t="n">
+        <v>23</v>
+      </c>
+      <c r="B8114" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8115">
+      <c r="A8115" t="n">
+        <v>23.33333333333333</v>
+      </c>
+      <c r="B8115" t="n">
+        <v>23.33333333333333</v>
+      </c>
+    </row>
+    <row r="8116">
+      <c r="A8116" t="n">
+        <v>23.33333333333333</v>
+      </c>
+      <c r="B8116" t="n">
+        <v>23.33333333333333</v>
+      </c>
+    </row>
+    <row r="8117">
+      <c r="A8117" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="B8117" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="8118">
+      <c r="A8118" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="B8118" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="8119">
+      <c r="A8119" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="B8119" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="8120">
+      <c r="A8120" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="B8120" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="8121">
+      <c r="A8121" t="n">
+        <v>24.14285714285714</v>
+      </c>
+      <c r="B8121" t="n">
+        <v>24.14285714285714</v>
+      </c>
+    </row>
+    <row r="8122">
+      <c r="A8122" t="n">
+        <v>24.14285714285714</v>
+      </c>
+      <c r="B8122" t="n">
+        <v>24.14285714285714</v>
+      </c>
+    </row>
+    <row r="8123">
+      <c r="A8123" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="B8123" t="n">
+        <v>24.25</v>
+      </c>
+    </row>
+    <row r="8124">
+      <c r="A8124" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="B8124" t="n">
+        <v>24.25</v>
+      </c>
+    </row>
+    <row r="8125">
+      <c r="A8125" t="n">
+        <v>24.44444444444444</v>
+      </c>
+      <c r="B8125" t="n">
+        <v>24.44444444444444</v>
+      </c>
+    </row>
+    <row r="8126">
+      <c r="A8126" t="n">
+        <v>24.44444444444444</v>
+      </c>
+      <c r="B8126" t="n">
+        <v>24.44444444444444</v>
+      </c>
+    </row>
+    <row r="8127">
+      <c r="A8127" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="B8127" t="n">
+        <v>24.6</v>
+      </c>
+    </row>
+    <row r="8128">
+      <c r="A8128" t="n">
+        <v>24.81818181818182</v>
+      </c>
+      <c r="B8128" t="n">
+        <v>24.81818181818182</v>
+      </c>
+    </row>
+    <row r="8129">
+      <c r="A8129" t="n">
+        <v>24.81818181818182</v>
+      </c>
+      <c r="B8129" t="n">
+        <v>24.81818181818182</v>
+      </c>
+    </row>
+    <row r="8130">
+      <c r="A8130" t="n">
+        <v>25.08333333333333</v>
+      </c>
+      <c r="B8130" t="n">
+        <v>25.08333333333333</v>
+      </c>
+    </row>
+    <row r="8131">
+      <c r="A8131" t="n">
+        <v>25.38461538461538</v>
+      </c>
+      <c r="B8131" t="n">
+        <v>25.38461538461538</v>
+      </c>
+    </row>
+    <row r="8132">
+      <c r="A8132" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="B8132" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="8133">
+      <c r="A8133" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="B8133" t="n">
+        <v>25.75</v>
+      </c>
+    </row>
+    <row r="8134">
+      <c r="A8134" t="n">
+        <v>25.75</v>
+      </c>
+      <c r="B8134" t="n">
+        <v>25.75</v>
+      </c>
+    </row>
+    <row r="8135">
+      <c r="A8135" t="n">
+        <v>25.76470588235294</v>
+      </c>
+      <c r="B8135" t="n">
+        <v>25.76470588235294</v>
+      </c>
+    </row>
+    <row r="8136">
+      <c r="A8136" t="n">
+        <v>25.83333333333333</v>
+      </c>
+      <c r="B8136" t="n">
+        <v>25.83333333333333</v>
+      </c>
+    </row>
+    <row r="8137">
+      <c r="A8137" t="n">
+        <v>25.94736842105263</v>
+      </c>
+      <c r="B8137" t="n">
+        <v>25.94736842105263</v>
+      </c>
+    </row>
+    <row r="8138">
+      <c r="A8138" t="n">
+        <v>25.90476190476191</v>
+      </c>
+      <c r="B8138" t="n">
+        <v>25.90476190476191</v>
+      </c>
+    </row>
+    <row r="8139">
+      <c r="A8139" t="n">
+        <v>25.90476190476191</v>
+      </c>
+      <c r="B8139" t="n">
+        <v>25.90476190476191</v>
+      </c>
+    </row>
+    <row r="8140">
+      <c r="A8140" t="n">
+        <v>25.8695652173913</v>
+      </c>
+      <c r="B8140" t="n">
+        <v>25.8695652173913</v>
+      </c>
+    </row>
+    <row r="8141">
+      <c r="A8141" t="n">
+        <v>25.8695652173913</v>
+      </c>
+      <c r="B8141" t="n">
+        <v>25.8695652173913</v>
+      </c>
+    </row>
+    <row r="8142">
+      <c r="A8142" t="n">
+        <v>25.91666666666667</v>
+      </c>
+      <c r="B8142" t="n">
+        <v>25.91666666666667</v>
+      </c>
+    </row>
+    <row r="8143">
+      <c r="A8143" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="B8143" t="n">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="8144">
+      <c r="A8144" t="n">
+        <v>25.69230769230769</v>
+      </c>
+      <c r="B8144" t="n">
+        <v>25.69230769230769</v>
+      </c>
+    </row>
+    <row r="8145">
+      <c r="A8145" t="n">
+        <v>25.69230769230769</v>
+      </c>
+      <c r="B8145" t="n">
+        <v>25.69230769230769</v>
+      </c>
+    </row>
+    <row r="8146">
+      <c r="A8146" t="n">
+        <v>25.81481481481481</v>
+      </c>
+      <c r="B8146" t="n">
+        <v>25.81481481481481</v>
+      </c>
+    </row>
+    <row r="8147">
+      <c r="A8147" t="n">
+        <v>25.81481481481481</v>
+      </c>
+      <c r="B8147" t="n">
+        <v>25.81481481481481</v>
+      </c>
+    </row>
+    <row r="8148">
+      <c r="A8148" t="n">
+        <v>25.81481481481481</v>
+      </c>
+      <c r="B8148" t="n">
+        <v>25.81481481481481</v>
+      </c>
+    </row>
+    <row r="8149">
+      <c r="A8149" t="n">
+        <v>25.81481481481481</v>
+      </c>
+      <c r="B8149" t="n">
+        <v>25.81481481481481</v>
+      </c>
+    </row>
+    <row r="8150">
+      <c r="A8150" t="n">
+        <v>25.81481481481481</v>
+      </c>
+      <c r="B8150" t="n">
+        <v>25.81481481481481</v>
+      </c>
+    </row>
+    <row r="8151">
+      <c r="A8151" t="n">
+        <v>25.93103448275862</v>
+      </c>
+      <c r="B8151" t="n">
+        <v>25.93103448275862</v>
+      </c>
+    </row>
+    <row r="8152">
+      <c r="A8152" t="n">
+        <v>26.2258064516129</v>
+      </c>
+      <c r="B8152" t="n">
+        <v>26.2258064516129</v>
+      </c>
+    </row>
+    <row r="8153">
+      <c r="A8153" t="n">
+        <v>26.21212121212121</v>
+      </c>
+      <c r="B8153" t="n">
+        <v>26.21212121212121</v>
+      </c>
+    </row>
+    <row r="8154">
+      <c r="A8154" t="n">
+        <v>26.29411764705882</v>
+      </c>
+      <c r="B8154" t="n">
+        <v>26.29411764705882</v>
+      </c>
+    </row>
+    <row r="8155">
+      <c r="A8155" t="n">
+        <v>26.29411764705882</v>
+      </c>
+      <c r="B8155" t="n">
+        <v>26.29411764705882</v>
+      </c>
+    </row>
+    <row r="8156">
+      <c r="A8156" t="n">
+        <v>26.22857142857143</v>
+      </c>
+      <c r="B8156" t="n">
+        <v>26.22857142857143</v>
+      </c>
+    </row>
+    <row r="8157">
+      <c r="A8157" t="n">
+        <v>26.22857142857143</v>
+      </c>
+      <c r="B8157" t="n">
+        <v>26.22857142857143</v>
+      </c>
+    </row>
+    <row r="8158">
+      <c r="A8158" t="n">
+        <v>26.16666666666667</v>
+      </c>
+      <c r="B8158" t="n">
+        <v>26.16666666666667</v>
+      </c>
+    </row>
+    <row r="8159">
+      <c r="A8159" t="n">
+        <v>26.16666666666667</v>
+      </c>
+      <c r="B8159" t="n">
+        <v>26.16666666666667</v>
+      </c>
+    </row>
+    <row r="8160">
+      <c r="A8160" t="n">
+        <v>26.21621621621622</v>
+      </c>
+      <c r="B8160" t="n">
+        <v>26.21621621621622</v>
+      </c>
+    </row>
+    <row r="8161">
+      <c r="A8161" t="n">
+        <v>26.15789473684211</v>
+      </c>
+      <c r="B8161" t="n">
+        <v>26.15789473684211</v>
+      </c>
+    </row>
+    <row r="8162">
+      <c r="A8162" t="n">
+        <v>26.33333333333333</v>
+      </c>
+      <c r="B8162" t="n">
+        <v>26.33333333333333</v>
+      </c>
+    </row>
+    <row r="8163">
+      <c r="A8163" t="n">
+        <v>26.33333333333333</v>
+      </c>
+      <c r="B8163" t="n">
+        <v>26.33333333333333</v>
+      </c>
+    </row>
+    <row r="8164">
+      <c r="A8164" t="n">
+        <v>26.33333333333333</v>
+      </c>
+      <c r="B8164" t="n">
+        <v>26.33333333333333</v>
+      </c>
+    </row>
+    <row r="8165">
+      <c r="A8165" t="n">
+        <v>26.33333333333333</v>
+      </c>
+      <c r="B8165" t="n">
+        <v>26.33333333333333</v>
+      </c>
+    </row>
+    <row r="8166">
+      <c r="A8166" t="n">
+        <v>26.325</v>
+      </c>
+      <c r="B8166" t="n">
+        <v>26.325</v>
+      </c>
+    </row>
+    <row r="8167">
+      <c r="A8167" t="n">
+        <v>26.30952380952381</v>
+      </c>
+      <c r="B8167" t="n">
+        <v>26.30952380952381</v>
+      </c>
+    </row>
+    <row r="8168">
+      <c r="A8168" t="n">
+        <v>26.34883720930232</v>
+      </c>
+      <c r="B8168" t="n">
+        <v>26.34883720930232</v>
+      </c>
+    </row>
+    <row r="8169">
+      <c r="A8169" t="n">
+        <v>26.34883720930232</v>
+      </c>
+      <c r="B8169" t="n">
+        <v>26.34883720930232</v>
+      </c>
+    </row>
+    <row r="8170">
+      <c r="A8170" t="n">
+        <v>26.31818181818182</v>
+      </c>
+      <c r="B8170" t="n">
+        <v>26.31818181818182</v>
+      </c>
+    </row>
+    <row r="8171">
+      <c r="A8171" t="n">
+        <v>26.31818181818182</v>
+      </c>
+      <c r="B8171" t="n">
+        <v>26.31818181818182</v>
+      </c>
+    </row>
+    <row r="8172">
+      <c r="A8172" t="n">
+        <v>26.42222222222222</v>
+      </c>
+      <c r="B8172" t="n">
+        <v>26.34782608695652</v>
+      </c>
+    </row>
+    <row r="8173">
+      <c r="A8173" t="n">
+        <v>26.44444444444444</v>
+      </c>
+      <c r="B8173" t="n">
+        <v>26.29787234042553</v>
+      </c>
+    </row>
+    <row r="8174">
+      <c r="A8174" t="n">
+        <v>26.41304347826087</v>
+      </c>
+      <c r="B8174" t="n">
+        <v>26.27083333333333</v>
+      </c>
+    </row>
+    <row r="8175">
+      <c r="A8175" t="n">
+        <v>26.46666666666667</v>
+      </c>
+      <c r="B8175" t="n">
+        <v>26.27083333333333</v>
+      </c>
+    </row>
+    <row r="8176">
+      <c r="A8176" t="n">
+        <v>26.43478260869565</v>
+      </c>
+      <c r="B8176" t="n">
+        <v>26.24489795918367</v>
+      </c>
+    </row>
+    <row r="8177">
+      <c r="A8177" t="n">
+        <v>26.47826086956522</v>
+      </c>
+      <c r="B8177" t="n">
+        <v>26.24</v>
+      </c>
+    </row>
+    <row r="8178">
+      <c r="A8178" t="n">
+        <v>26.47826086956522</v>
+      </c>
+      <c r="B8178" t="n">
+        <v>26.24</v>
+      </c>
+    </row>
+    <row r="8179">
+      <c r="A8179" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="B8179" t="n">
+        <v>26.23529411764706</v>
+      </c>
+    </row>
+    <row r="8180">
+      <c r="A8180" t="n">
+        <v>26.46808510638298</v>
+      </c>
+      <c r="B8180" t="n">
+        <v>26.21153846153846</v>
+      </c>
+    </row>
+    <row r="8181">
+      <c r="A8181" t="n">
+        <v>26.48936170212766</v>
+      </c>
+      <c r="B8181" t="n">
+        <v>26.18518518518519</v>
+      </c>
+    </row>
+    <row r="8182">
+      <c r="A8182" t="n">
+        <v>26.48936170212766</v>
+      </c>
+      <c r="B8182" t="n">
+        <v>26.18518518518519</v>
+      </c>
+    </row>
+    <row r="8183">
+      <c r="A8183" t="n">
+        <v>26.52173913043478</v>
+      </c>
+      <c r="B8183" t="n">
+        <v>26.18518518518519</v>
+      </c>
+    </row>
+    <row r="8184">
+      <c r="A8184" t="n">
+        <v>26.48936170212766</v>
+      </c>
+      <c r="B8184" t="n">
+        <v>26.16363636363636</v>
+      </c>
+    </row>
+    <row r="8185">
+      <c r="A8185" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="B8185" t="n">
+        <v>26.16363636363636</v>
+      </c>
+    </row>
+    <row r="8186">
+      <c r="A8186" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="B8186" t="n">
+        <v>26.16363636363636</v>
+      </c>
+    </row>
+    <row r="8187">
+      <c r="A8187" t="n">
+        <v>26.57446808510638</v>
+      </c>
+      <c r="B8187" t="n">
+        <v>26.2280701754386</v>
+      </c>
+    </row>
+    <row r="8188">
+      <c r="A8188" t="n">
+        <v>26.56521739130435</v>
+      </c>
+      <c r="B8188" t="n">
+        <v>26.2280701754386</v>
+      </c>
+    </row>
+    <row r="8189">
+      <c r="A8189" t="n">
+        <v>26.56521739130435</v>
+      </c>
+      <c r="B8189" t="n">
+        <v>26.2280701754386</v>
+      </c>
+    </row>
+    <row r="8190">
+      <c r="A8190" t="n">
+        <v>26.59574468085106</v>
+      </c>
+      <c r="B8190" t="n">
+        <v>26.28813559322034</v>
+      </c>
+    </row>
+    <row r="8191">
+      <c r="A8191" t="n">
+        <v>26.53191489361702</v>
+      </c>
+      <c r="B8191" t="n">
+        <v>26.28333333333333</v>
+      </c>
+    </row>
+    <row r="8192">
+      <c r="A8192" t="n">
+        <v>26.42857142857143</v>
+      </c>
+      <c r="B8192" t="n">
+        <v>26.22222222222222</v>
+      </c>
+    </row>
+    <row r="8193">
+      <c r="A8193" t="n">
+        <v>26.38297872340426</v>
+      </c>
+      <c r="B8193" t="n">
+        <v>26.22222222222222</v>
+      </c>
+    </row>
+    <row r="8194">
+      <c r="A8194" t="n">
+        <v>26.38297872340426</v>
+      </c>
+      <c r="B8194" t="n">
+        <v>26.22222222222222</v>
+      </c>
+    </row>
+    <row r="8195">
+      <c r="A8195" t="n">
+        <v>26.39130434782609</v>
+      </c>
+      <c r="B8195" t="n">
+        <v>26.22222222222222</v>
+      </c>
+    </row>
+    <row r="8196">
+      <c r="A8196" t="n">
+        <v>26.32608695652174</v>
+      </c>
+      <c r="B8196" t="n">
+        <v>26.1875</v>
+      </c>
+    </row>
+    <row r="8197">
+      <c r="A8197" t="n">
+        <v>26.36170212765957</v>
+      </c>
+      <c r="B8197" t="n">
+        <v>26.24242424242424</v>
+      </c>
+    </row>
+    <row r="8198">
+      <c r="A8198" t="n">
+        <v>26.52173913043478</v>
+      </c>
+      <c r="B8198" t="n">
+        <v>26.32835820895522</v>
+      </c>
+    </row>
+    <row r="8199">
+      <c r="A8199" t="n">
+        <v>26.59574468085106</v>
+      </c>
+      <c r="B8199" t="n">
+        <v>26.38235294117647</v>
+      </c>
+    </row>
+    <row r="8200">
+      <c r="A8200" t="n">
+        <v>26.60869565217391</v>
+      </c>
+      <c r="B8200" t="n">
+        <v>26.36231884057971</v>
+      </c>
+    </row>
+    <row r="8201">
+      <c r="A8201" t="n">
+        <v>26.60416666666667</v>
+      </c>
+      <c r="B8201" t="n">
+        <v>26.36619718309859</v>
+      </c>
+    </row>
+    <row r="8202">
+      <c r="A8202" t="n">
+        <v>26.59574468085106</v>
+      </c>
+      <c r="B8202" t="n">
+        <v>26.36619718309859</v>
+      </c>
+    </row>
+    <row r="8203">
+      <c r="A8203" t="n">
+        <v>26.67391304347826</v>
+      </c>
+      <c r="B8203" t="n">
+        <v>26.36619718309859</v>
+      </c>
+    </row>
+    <row r="8204">
+      <c r="A8204" t="n">
+        <v>26.75555555555556</v>
+      </c>
+      <c r="B8204" t="n">
+        <v>26.36619718309859</v>
+      </c>
+    </row>
+    <row r="8205">
+      <c r="A8205" t="n">
+        <v>26.76086956521739</v>
+      </c>
+      <c r="B8205" t="n">
+        <v>26.375</v>
+      </c>
+    </row>
+    <row r="8206">
+      <c r="A8206" t="n">
+        <v>26.78260869565218</v>
+      </c>
+      <c r="B8206" t="n">
+        <v>26.42465753424657</v>
+      </c>
+    </row>
+    <row r="8207">
+      <c r="A8207" t="n">
+        <v>26.95744680851064</v>
+      </c>
+      <c r="B8207" t="n">
+        <v>26.54054054054054</v>
+      </c>
+    </row>
+    <row r="8208">
+      <c r="A8208" t="n">
+        <v>26.93877551020408</v>
+      </c>
+      <c r="B8208" t="n">
+        <v>26.53947368421053</v>
+      </c>
+    </row>
+    <row r="8209">
+      <c r="A8209" t="n">
+        <v>26.93877551020408</v>
+      </c>
+      <c r="B8209" t="n">
+        <v>26.53947368421053</v>
+      </c>
+    </row>
+    <row r="8210">
+      <c r="A8210" t="n">
+        <v>26.92</v>
+      </c>
+      <c r="B8210" t="n">
+        <v>26.53246753246753</v>
+      </c>
+    </row>
+    <row r="8211">
+      <c r="A8211" t="n">
+        <v>26.89795918367347</v>
+      </c>
+      <c r="B8211" t="n">
+        <v>26.53846153846154</v>
+      </c>
+    </row>
+    <row r="8212">
+      <c r="A8212" t="n">
+        <v>26.89583333333333</v>
+      </c>
+      <c r="B8212" t="n">
+        <v>26.63291139240506</v>
+      </c>
+    </row>
+    <row r="8213">
+      <c r="A8213" t="n">
+        <v>26.87234042553191</v>
+      </c>
+      <c r="B8213" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="8214">
+      <c r="A8214" t="n">
+        <v>26.82608695652174</v>
+      </c>
+      <c r="B8214" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="8215">
+      <c r="A8215" t="n">
+        <v>26.82608695652174</v>
+      </c>
+      <c r="B8215" t="n">
+        <v>26.6</v>
+      </c>
+    </row>
+    <row r="8216">
+      <c r="A8216" t="n">
+        <v>26.80434782608696</v>
+      </c>
+      <c r="B8216" t="n">
+        <v>26.55555555555556</v>
+      </c>
+    </row>
+    <row r="8217">
+      <c r="A8217" t="n">
+        <v>26.80434782608696</v>
+      </c>
+      <c r="B8217" t="n">
+        <v>26.55555555555556</v>
+      </c>
+    </row>
+    <row r="8218">
+      <c r="A8218" t="n">
+        <v>27.02127659574468</v>
+      </c>
+      <c r="B8218" t="n">
+        <v>26.65060240963856</v>
+      </c>
+    </row>
+    <row r="8219">
+      <c r="A8219" t="n">
+        <v>27.02127659574468</v>
+      </c>
+      <c r="B8219" t="n">
+        <v>26.65060240963856</v>
+      </c>
+    </row>
+    <row r="8220">
+      <c r="A8220" t="n">
+        <v>27.17021276595745</v>
+      </c>
+      <c r="B8220" t="n">
+        <v>26.75</v>
+      </c>
+    </row>
+    <row r="8221">
+      <c r="A8221" t="n">
+        <v>27.23913043478261</v>
+      </c>
+      <c r="B8221" t="n">
+        <v>26.75</v>
+      </c>
+    </row>
+    <row r="8222">
+      <c r="A8222" t="n">
+        <v>27.21276595744681</v>
+      </c>
+      <c r="B8222" t="n">
+        <v>26.81395348837209</v>
+      </c>
+    </row>
+    <row r="8223">
+      <c r="A8223" t="n">
+        <v>27.21276595744681</v>
+      </c>
+      <c r="B8223" t="n">
+        <v>26.81395348837209</v>
+      </c>
+    </row>
+    <row r="8224">
+      <c r="A8224" t="n">
+        <v>27.21276595744681</v>
+      </c>
+      <c r="B8224" t="n">
+        <v>26.81395348837209</v>
+      </c>
+    </row>
+    <row r="8225">
+      <c r="A8225" t="n">
+        <v>27.16666666666667</v>
+      </c>
+      <c r="B8225" t="n">
+        <v>26.79310344827586</v>
+      </c>
+    </row>
+    <row r="8226">
+      <c r="A8226" t="n">
+        <v>27.19148936170213</v>
+      </c>
+      <c r="B8226" t="n">
+        <v>26.79310344827586</v>
+      </c>
+    </row>
+    <row r="8227">
+      <c r="A8227" t="n">
+        <v>27.24444444444444</v>
+      </c>
+      <c r="B8227" t="n">
+        <v>26.79310344827586</v>
+      </c>
+    </row>
+    <row r="8228">
+      <c r="A8228" t="n">
+        <v>27.22727272727273</v>
+      </c>
+      <c r="B8228" t="n">
+        <v>26.79310344827586</v>
+      </c>
+    </row>
+    <row r="8229">
+      <c r="A8229" t="n">
+        <v>27.22727272727273</v>
+      </c>
+      <c r="B8229" t="n">
+        <v>26.79310344827586</v>
+      </c>
+    </row>
+    <row r="8230">
+      <c r="A8230" t="n">
+        <v>27.27906976744186</v>
+      </c>
+      <c r="B8230" t="n">
+        <v>26.79310344827586</v>
+      </c>
+    </row>
+    <row r="8231">
+      <c r="A8231" t="n">
+        <v>27.27272727272727</v>
+      </c>
+      <c r="B8231" t="n">
+        <v>26.79545454545455</v>
+      </c>
+    </row>
+    <row r="8232">
+      <c r="A8232" t="n">
+        <v>27.28571428571428</v>
+      </c>
+      <c r="B8232" t="n">
+        <v>26.79545454545455</v>
+      </c>
+    </row>
+    <row r="8233">
+      <c r="A8233" t="n">
+        <v>27.32558139534884</v>
+      </c>
+      <c r="B8233" t="n">
+        <v>26.78888888888889</v>
+      </c>
+    </row>
+    <row r="8234">
+      <c r="A8234" t="n">
+        <v>27.47727272727273</v>
+      </c>
+      <c r="B8234" t="n">
+        <v>26.84782608695652</v>
+      </c>
+    </row>
+    <row r="8235">
+      <c r="A8235" t="n">
+        <v>27.47727272727273</v>
+      </c>
+      <c r="B8235" t="n">
+        <v>26.84782608695652</v>
+      </c>
+    </row>
+    <row r="8236">
+      <c r="A8236" t="n">
+        <v>27.53488372093023</v>
+      </c>
+      <c r="B8236" t="n">
+        <v>26.84782608695652</v>
+      </c>
+    </row>
+    <row r="8237">
+      <c r="A8237" t="n">
+        <v>27.57142857142857</v>
+      </c>
+      <c r="B8237" t="n">
+        <v>26.84782608695652</v>
+      </c>
+    </row>
+    <row r="8238">
+      <c r="A8238" t="n">
+        <v>27.57142857142857</v>
+      </c>
+      <c r="B8238" t="n">
+        <v>26.84782608695652</v>
+      </c>
+    </row>
+    <row r="8239">
+      <c r="A8239" t="n">
+        <v>27.59523809523809</v>
+      </c>
+      <c r="B8239" t="n">
+        <v>26.8494623655914</v>
+      </c>
+    </row>
+    <row r="8240">
+      <c r="A8240" t="n">
+        <v>27.57142857142857</v>
+      </c>
+      <c r="B8240" t="n">
+        <v>26.81914893617021</v>
+      </c>
+    </row>
+    <row r="8241">
+      <c r="A8241" t="n">
+        <v>27.675</v>
+      </c>
+      <c r="B8241" t="n">
+        <v>26.81914893617021</v>
+      </c>
+    </row>
+    <row r="8242">
+      <c r="A8242" t="n">
+        <v>27.5609756097561</v>
+      </c>
+      <c r="B8242" t="n">
+        <v>26.77894736842105</v>
+      </c>
+    </row>
+    <row r="8243">
+      <c r="A8243" t="n">
+        <v>27.5609756097561</v>
+      </c>
+      <c r="B8243" t="n">
+        <v>26.77894736842105</v>
+      </c>
+    </row>
+    <row r="8244">
+      <c r="A8244" t="n">
+        <v>27.625</v>
+      </c>
+      <c r="B8244" t="n">
+        <v>26.77894736842105</v>
+      </c>
+    </row>
+    <row r="8245">
+      <c r="A8245" t="n">
+        <v>27.625</v>
+      </c>
+      <c r="B8245" t="n">
+        <v>26.77894736842105</v>
+      </c>
+    </row>
+    <row r="8246">
+      <c r="A8246" t="n">
+        <v>27.53658536585366</v>
+      </c>
+      <c r="B8246" t="n">
+        <v>26.75</v>
+      </c>
+    </row>
+    <row r="8247">
+      <c r="A8247" t="n">
+        <v>27.675</v>
+      </c>
+      <c r="B8247" t="n">
+        <v>26.82474226804124</v>
+      </c>
+    </row>
+    <row r="8248">
+      <c r="A8248" t="n">
+        <v>27.675</v>
+      </c>
+      <c r="B8248" t="n">
+        <v>26.82474226804124</v>
+      </c>
+    </row>
+    <row r="8249">
+      <c r="A8249" t="n">
+        <v>27.675</v>
+      </c>
+      <c r="B8249" t="n">
+        <v>26.82474226804124</v>
+      </c>
+    </row>
+    <row r="8250">
+      <c r="A8250" t="n">
+        <v>27.65789473684211</v>
+      </c>
+      <c r="B8250" t="n">
+        <v>26.82474226804124</v>
+      </c>
+    </row>
+    <row r="8251">
+      <c r="A8251" t="n">
+        <v>27.7027027027027</v>
+      </c>
+      <c r="B8251" t="n">
+        <v>26.82474226804124</v>
+      </c>
+    </row>
+    <row r="8252">
+      <c r="A8252" t="n">
+        <v>27.88571428571429</v>
+      </c>
+      <c r="B8252" t="n">
+        <v>26.81632653061224</v>
+      </c>
+    </row>
+    <row r="8253">
+      <c r="A8253" t="n">
+        <v>27.88571428571429</v>
+      </c>
+      <c r="B8253" t="n">
+        <v>26.81632653061224</v>
+      </c>
+    </row>
+    <row r="8254">
+      <c r="A8254" t="n">
+        <v>27.81081081081081</v>
+      </c>
+      <c r="B8254" t="n">
+        <v>26.81</v>
+      </c>
+    </row>
+    <row r="8255">
+      <c r="A8255" t="n">
+        <v>27.81081081081081</v>
+      </c>
+      <c r="B8255" t="n">
+        <v>26.81</v>
+      </c>
+    </row>
+    <row r="8256">
+      <c r="A8256" t="n">
+        <v>27.71052631578947</v>
+      </c>
+      <c r="B8256" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8257">
+      <c r="A8257" t="n">
+        <v>27.69444444444444</v>
+      </c>
+      <c r="B8257" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8258">
+      <c r="A8258" t="n">
+        <v>27.57142857142857</v>
+      </c>
+      <c r="B8258" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8259">
+      <c r="A8259" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="B8259" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8260">
+      <c r="A8260" t="n">
+        <v>27.57575757575757</v>
+      </c>
+      <c r="B8260" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8261">
+      <c r="A8261" t="n">
+        <v>27.64516129032258</v>
+      </c>
+      <c r="B8261" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8262">
+      <c r="A8262" t="n">
+        <v>27.64516129032258</v>
+      </c>
+      <c r="B8262" t="n">
+        <v>26.75490196078431</v>
+      </c>
+    </row>
+    <row r="8263">
+      <c r="A8263" t="n">
+        <v>27.51515151515152</v>
+      </c>
+      <c r="B8263" t="n">
+        <v>26.73076923076923</v>
+      </c>
+    </row>
+    <row r="8264">
+      <c r="A8264" t="n">
+        <v>27.51515151515152</v>
+      </c>
+      <c r="B8264" t="n">
+        <v>26.73076923076923</v>
+      </c>
+    </row>
+    <row r="8265">
+      <c r="A8265" t="n">
+        <v>27.45454545454545</v>
+      </c>
+      <c r="B8265" t="n">
+        <v>26.71428571428572</v>
+      </c>
+    </row>
+    <row r="8266">
+      <c r="A8266" t="n">
+        <v>27.375</v>
+      </c>
+      <c r="B8266" t="n">
+        <v>26.71428571428572</v>
+      </c>
+    </row>
+    <row r="8267">
+      <c r="A8267" t="n">
+        <v>27.12903225806452</v>
+      </c>
+      <c r="B8267" t="n">
+        <v>26.71428571428572</v>
+      </c>
+    </row>
+    <row r="8268">
+      <c r="A8268" t="n">
+        <v>27.17241379310345</v>
+      </c>
+      <c r="B8268" t="n">
+        <v>26.71428571428572</v>
+      </c>
+    </row>
+    <row r="8269">
+      <c r="A8269" t="n">
+        <v>27.17241379310345</v>
+      </c>
+      <c r="B8269" t="n">
+        <v>26.71428571428572</v>
+      </c>
+    </row>
+    <row r="8270">
+      <c r="A8270" t="n">
+        <v>27.20689655172414</v>
+      </c>
+      <c r="B8270" t="n">
+        <v>26.71698113207547</v>
+      </c>
+    </row>
+    <row r="8271">
+      <c r="A8271" t="n">
+        <v>27.21428571428572</v>
+      </c>
+      <c r="B8271" t="n">
+        <v>26.71698113207547</v>
+      </c>
+    </row>
+    <row r="8272">
+      <c r="A8272" t="n">
+        <v>26.89285714285714</v>
+      </c>
+      <c r="B8272" t="n">
+        <v>26.70093457943925</v>
+      </c>
+    </row>
+    <row r="8273">
+      <c r="A8273" t="n">
+        <v>27</v>
+      </c>
+      <c r="B8273" t="n">
+        <v>26.70093457943925</v>
+      </c>
+    </row>
+    <row r="8274">
+      <c r="A8274" t="n">
+        <v>26.89655172413793</v>
+      </c>
+      <c r="B8274" t="n">
+        <v>26.67889908256881</v>
+      </c>
+    </row>
+    <row r="8275">
+      <c r="A8275" t="n">
+        <v>26.89655172413793</v>
+      </c>
+      <c r="B8275" t="n">
+        <v>26.67889908256881</v>
+      </c>
+    </row>
+    <row r="8276">
+      <c r="A8276" t="n">
+        <v>27.03571428571428</v>
+      </c>
+      <c r="B8276" t="n">
+        <v>26.67889908256881</v>
+      </c>
+    </row>
+    <row r="8277">
+      <c r="A8277" t="n">
+        <v>27.03571428571428</v>
+      </c>
+      <c r="B8277" t="n">
+        <v>26.67889908256881</v>
+      </c>
+    </row>
+    <row r="8278">
+      <c r="A8278" t="n">
+        <v>26.76923076923077</v>
+      </c>
+      <c r="B8278" t="n">
+        <v>26.67889908256881</v>
+      </c>
+    </row>
+    <row r="8279">
+      <c r="A8279" t="n">
+        <v>26.76923076923077</v>
+      </c>
+      <c r="B8279" t="n">
+        <v>26.67889908256881</v>
+      </c>
+    </row>
+    <row r="8280">
+      <c r="A8280" t="n">
+        <v>26.46153846153846</v>
+      </c>
+      <c r="B8280" t="n">
+        <v>26.68181818181818</v>
+      </c>
+    </row>
+    <row r="8281">
+      <c r="A8281" t="n">
+        <v>26.44444444444444</v>
+      </c>
+      <c r="B8281" t="n">
+        <v>26.67567567567568</v>
+      </c>
+    </row>
+    <row r="8282">
+      <c r="A8282" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="B8282" t="n">
+        <v>26.67567567567568</v>
+      </c>
+    </row>
+    <row r="8283">
+      <c r="A8283" t="n">
+        <v>26.07407407407407</v>
+      </c>
+      <c r="B8283" t="n">
+        <v>26.63716814159292</v>
+      </c>
+    </row>
+    <row r="8284">
+      <c r="A8284" t="n">
+        <v>26</v>
+      </c>
+      <c r="B8284" t="n">
+        <v>26.6140350877193</v>
+      </c>
+    </row>
+    <row r="8285">
+      <c r="A8285" t="n">
+        <v>26.03703703703704</v>
+      </c>
+      <c r="B8285" t="n">
+        <v>26.6140350877193</v>
+      </c>
+    </row>
+    <row r="8286">
+      <c r="A8286" t="n">
+        <v>26.03703703703704</v>
+      </c>
+      <c r="B8286" t="n">
+        <v>26.6140350877193</v>
+      </c>
+    </row>
+    <row r="8287">
+      <c r="A8287" t="n">
+        <v>25.96428571428572</v>
+      </c>
+      <c r="B8287" t="n">
+        <v>26.59130434782609</v>
+      </c>
+    </row>
+    <row r="8288">
+      <c r="A8288" t="n">
+        <v>25.96428571428572</v>
+      </c>
+      <c r="B8288" t="n">
+        <v>26.59130434782609</v>
+      </c>
+    </row>
+    <row r="8289">
+      <c r="A8289" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="B8289" t="n">
+        <v>26.56410256410257</v>
+      </c>
+    </row>
+    <row r="8290">
+      <c r="A8290" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="B8290" t="n">
+        <v>26.56410256410257</v>
+      </c>
+    </row>
+    <row r="8291">
+      <c r="A8291" t="n">
+        <v>25.86206896551724</v>
+      </c>
+      <c r="B8291" t="n">
+        <v>26.56410256410257</v>
+      </c>
+    </row>
+    <row r="8292">
+      <c r="A8292" t="n">
+        <v>25.86206896551724</v>
+      </c>
+      <c r="B8292" t="n">
+        <v>26.56410256410257</v>
+      </c>
+    </row>
+    <row r="8293">
+      <c r="A8293" t="n">
+        <v>25.81481481481481</v>
+      </c>
+      <c r="B8293" t="n">
+        <v>26.56410256410257</v>
+      </c>
+    </row>
+    <row r="8294">
+      <c r="A8294" t="n">
+        <v>25.51851851851852</v>
+      </c>
+      <c r="B8294" t="n">
+        <v>26.54621848739496</v>
+      </c>
+    </row>
+    <row r="8295">
+      <c r="A8295" t="n">
+        <v>25.51851851851852</v>
+      </c>
+      <c r="B8295" t="n">
+        <v>26.54621848739496</v>
+      </c>
+    </row>
+    <row r="8296">
+      <c r="A8296" t="n">
+        <v>25.64285714285714</v>
+      </c>
+      <c r="B8296" t="n">
+        <v>26.56666666666667</v>
+      </c>
+    </row>
+    <row r="8297">
+      <c r="A8297" t="n">
+        <v>25.64285714285714</v>
+      </c>
+      <c r="B8297" t="n">
+        <v>26.56666666666667</v>
+      </c>
+    </row>
+    <row r="8298">
+      <c r="A8298" t="n">
+        <v>25.64285714285714</v>
+      </c>
+      <c r="B8298" t="n">
+        <v>26.56666666666667</v>
+      </c>
+    </row>
+    <row r="8299">
+      <c r="A8299" t="n">
+        <v>25.59259259259259</v>
+      </c>
+      <c r="B8299" t="n">
+        <v>26.56666666666667</v>
+      </c>
+    </row>
+    <row r="8300">
+      <c r="A8300" t="n">
+        <v>25.57142857142857</v>
+      </c>
+      <c r="B8300" t="n">
+        <v>26.5327868852459</v>
+      </c>
+    </row>
+    <row r="8301">
+      <c r="A8301" t="n">
+        <v>25.57142857142857</v>
+      </c>
+      <c r="B8301" t="n">
+        <v>26.5327868852459</v>
+      </c>
+    </row>
+    <row r="8302">
+      <c r="A8302" t="n">
+        <v>25.72413793103448</v>
+      </c>
+      <c r="B8302" t="n">
+        <v>26.53225806451613</v>
+      </c>
+    </row>
+    <row r="8303">
+      <c r="A8303" t="n">
+        <v>25.72413793103448</v>
+      </c>
+      <c r="B8303" t="n">
+        <v>26.53225806451613</v>
+      </c>
+    </row>
+    <row r="8304">
+      <c r="A8304" t="n">
+        <v>25.72413793103448</v>
+      </c>
+      <c r="B8304" t="n">
+        <v>26.53225806451613</v>
+      </c>
+    </row>
+    <row r="8305">
+      <c r="A8305" t="n">
+        <v>25.72413793103448</v>
+      </c>
+      <c r="B8305" t="n">
+        <v>26.53225806451613</v>
+      </c>
+    </row>
+    <row r="8306">
+      <c r="A8306" t="n">
+        <v>25.72413793103448</v>
+      </c>
+      <c r="B8306" t="n">
+        <v>26.512</v>
+      </c>
+    </row>
+    <row r="8307">
+      <c r="A8307" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="B8307" t="n">
+        <v>26.512</v>
+      </c>
+    </row>
+    <row r="8308">
+      <c r="A8308" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="B8308" t="n">
+        <v>26.512</v>
+      </c>
+    </row>
+    <row r="8309">
+      <c r="A8309" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="B8309" t="n">
+        <v>26.512</v>
+      </c>
+    </row>
+    <row r="8310">
+      <c r="A8310" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="B8310" t="n">
+        <v>26.512</v>
+      </c>
+    </row>
+    <row r="8311">
+      <c r="A8311" t="n">
+        <v>25.44827586206896</v>
+      </c>
+      <c r="B8311" t="n">
+        <v>26.50793650793651</v>
+      </c>
+    </row>
+    <row r="8312">
+      <c r="A8312" t="n">
+        <v>25.42857142857143</v>
+      </c>
+      <c r="B8312" t="n">
+        <v>26.50793650793651</v>
+      </c>
+    </row>
+    <row r="8313">
+      <c r="A8313" t="n">
+        <v>25.48275862068965</v>
+      </c>
+      <c r="B8313" t="n">
+        <v>26.51181102362205</v>
+      </c>
+    </row>
+    <row r="8314">
+      <c r="A8314" t="n">
+        <v>25.32142857142857</v>
+      </c>
+      <c r="B8314" t="n">
+        <v>26.484375</v>
+      </c>
+    </row>
+    <row r="8315">
+      <c r="A8315" t="n">
+        <v>25.32142857142857</v>
+      </c>
+      <c r="B8315" t="n">
+        <v>26.484375</v>
+      </c>
+    </row>
+    <row r="8316">
+      <c r="A8316" t="n">
+        <v>25.42307692307692</v>
+      </c>
+      <c r="B8316" t="n">
+        <v>26.484375</v>
+      </c>
+    </row>
+    <row r="8317">
+      <c r="A8317" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8317" t="n">
+        <v>26.45736434108527</v>
+      </c>
+    </row>
+    <row r="8318">
+      <c r="A8318" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8318" t="n">
+        <v>26.45736434108527</v>
+      </c>
+    </row>
+    <row r="8319">
+      <c r="A8319" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8319" t="n">
+        <v>26.45736434108527</v>
+      </c>
+    </row>
+    <row r="8320">
+      <c r="A8320" t="n">
+        <v>25.33333333333333</v>
+      </c>
+      <c r="B8320" t="n">
+        <v>26.45736434108527</v>
+      </c>
+    </row>
+    <row r="8321">
+      <c r="A8321" t="n">
+        <v>25.35714285714286</v>
+      </c>
+      <c r="B8321" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
+    <row r="8322">
+      <c r="A8322" t="n">
+        <v>25.35714285714286</v>
+      </c>
+      <c r="B8322" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
+    <row r="8323">
+      <c r="A8323" t="n">
+        <v>25.34615384615385</v>
+      </c>
+      <c r="B8323" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
+    <row r="8324">
+      <c r="A8324" t="n">
+        <v>25.34615384615385</v>
+      </c>
+      <c r="B8324" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
+    <row r="8325">
+      <c r="A8325" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="B8325" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
+    <row r="8326">
+      <c r="A8326" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="B8326" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
+    <row r="8327">
+      <c r="A8327" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="B8327" t="n">
+        <v>26.45384615384615</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>